<commit_message>
Updated BOM According to #8
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/Digikey_BOM.xlsx
+++ b/Documents/Deliverables/BOM/Digikey_BOM.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="275">
   <si>
     <t>S. No.</t>
   </si>
@@ -850,9 +850,6 @@
     <t xml:space="preserve">SG90 </t>
   </si>
   <si>
-    <t>Amazon</t>
-  </si>
-  <si>
     <t xml:space="preserve">Laod Cell </t>
   </si>
   <si>
@@ -863,6 +860,9 @@
   </si>
   <si>
     <t xml:space="preserve">SG90 Servo Motor, Micro Servo 9G SG90 Kit for RC Robot Arm/Walking Helicopter Airplane Car Boat Control, Micro Servos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TDK </t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1011,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1032,18 +1032,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -1387,34 +1381,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -1540,6 +1510,54 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1555,12 +1573,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1620,15 +1632,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1668,45 +1671,33 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1716,7 +1707,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1731,7 +1722,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1749,7 +1740,158 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1764,201 +1906,63 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="3" borderId="27" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" quotePrefix="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2247,2829 +2251,2881 @@
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="62.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="44.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="96" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="110"/>
-      <c r="C1" s="110"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="110"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="111"/>
+      <c r="B1" s="97"/>
+      <c r="C1" s="97"/>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+      <c r="P1" s="97"/>
+      <c r="Q1" s="98"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="68" t="s">
+      <c r="C2" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="68" t="s">
+      <c r="D2" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="68" t="s">
+      <c r="E2" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="68" t="s">
+      <c r="F2" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="68" t="s">
+      <c r="G2" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="68" t="s">
+      <c r="H2" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="68" t="s">
+      <c r="I2" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="68" t="s">
+      <c r="J2" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="68" t="s">
+      <c r="K2" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="68" t="s">
+      <c r="L2" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="68" t="s">
+      <c r="M2" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="68" t="s">
+      <c r="N2" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="68" t="s">
+      <c r="O2" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="68" t="s">
+      <c r="P2" s="59" t="s">
         <v>146</v>
       </c>
-      <c r="Q2" s="68" t="s">
+      <c r="Q2" s="59" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37">
+      <c r="A3" s="32">
         <v>1</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="106" t="s">
         <v>213</v>
       </c>
-      <c r="C3" s="90" t="s">
+      <c r="C3" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="69" t="s">
+      <c r="D3" s="60" t="s">
         <v>220</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="56" t="s">
+      <c r="H3" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="J3" s="18">
+      <c r="J3" s="16">
         <v>13</v>
       </c>
-      <c r="K3" s="17">
+      <c r="K3" s="15">
         <f>J3*5</f>
         <v>65</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M3" s="19">
+      <c r="M3" s="17">
         <v>0.03</v>
       </c>
-      <c r="N3" s="20">
+      <c r="N3" s="18">
         <f>M3*J3</f>
         <v>0.39</v>
       </c>
-      <c r="O3" s="19">
+      <c r="O3" s="17">
         <v>1.66E-2</v>
       </c>
-      <c r="P3" s="20">
+      <c r="P3" s="18">
         <f>O3*K3</f>
         <v>1.079</v>
       </c>
-      <c r="Q3" s="21"/>
+      <c r="Q3" s="19"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="37">
+      <c r="A4" s="32">
         <v>2</v>
       </c>
-      <c r="B4" s="126"/>
-      <c r="C4" s="34" t="s">
+      <c r="B4" s="107"/>
+      <c r="C4" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="63" t="s">
+      <c r="D4" s="54" t="s">
         <v>221</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="57" t="s">
+      <c r="H4" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="4">
         <v>7</v>
       </c>
-      <c r="K4" s="17">
+      <c r="K4" s="15">
         <f t="shared" ref="K4:K56" si="0">J4*5</f>
         <v>35</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M4" s="13">
+      <c r="M4" s="11">
         <v>0.1</v>
       </c>
-      <c r="N4" s="12">
+      <c r="N4" s="10">
         <f t="shared" ref="N4:N50" si="1">M4*J4</f>
         <v>0.70000000000000007</v>
       </c>
-      <c r="O4" s="13">
+      <c r="O4" s="11">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P4" s="12">
+      <c r="P4" s="10">
         <f t="shared" ref="P4:P50" si="2">O4*K4</f>
         <v>1.2250000000000001</v>
       </c>
-      <c r="Q4" s="7"/>
+      <c r="Q4" s="5"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37">
+      <c r="A5" s="32">
         <v>3</v>
       </c>
-      <c r="B5" s="126"/>
-      <c r="C5" s="34" t="s">
+      <c r="B5" s="107"/>
+      <c r="C5" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="54" t="s">
         <v>223</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="H5" s="57" t="s">
+      <c r="H5" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="4">
         <v>1</v>
       </c>
-      <c r="K5" s="17">
+      <c r="K5" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L5" s="92" t="s">
+      <c r="L5" s="76" t="s">
         <v>226</v>
       </c>
-      <c r="M5" s="91">
+      <c r="M5" s="75">
         <v>0.4</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="10">
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="O5" s="91">
+      <c r="O5" s="75">
         <v>0.4</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="10">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="Q5" s="7"/>
+      <c r="Q5" s="5"/>
     </row>
     <row r="6" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="37">
+      <c r="A6" s="32">
         <v>4</v>
       </c>
-      <c r="B6" s="126"/>
-      <c r="C6" s="34" t="s">
+      <c r="B6" s="107"/>
+      <c r="C6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="63" t="s">
+      <c r="D6" s="54" t="s">
         <v>227</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="128" t="s">
+      <c r="F6" s="91" t="s">
         <v>22</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="57" t="s">
+      <c r="H6" s="48" t="s">
         <v>219</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>6</v>
       </c>
-      <c r="K6" s="17">
+      <c r="K6" s="15">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="L6" s="89" t="s">
+      <c r="L6" s="73" t="s">
         <v>145</v>
       </c>
-      <c r="M6" s="13">
+      <c r="M6" s="11">
         <v>0.36</v>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="10">
         <f t="shared" si="1"/>
         <v>2.16</v>
       </c>
-      <c r="O6" s="13">
+      <c r="O6" s="11">
         <v>0.246</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="10">
         <f t="shared" si="2"/>
         <v>7.38</v>
       </c>
-      <c r="Q6" s="7"/>
+      <c r="Q6" s="5"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="37">
+      <c r="A7" s="32">
         <v>5</v>
       </c>
-      <c r="B7" s="126"/>
-      <c r="C7" s="34" t="s">
+      <c r="B7" s="107"/>
+      <c r="C7" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="D7" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="2" t="s">
         <v>26</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="57" t="s">
+      <c r="H7" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="4">
         <v>2</v>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M7" s="13">
+      <c r="M7" s="11">
         <v>0.39</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="10">
         <f t="shared" si="1"/>
         <v>0.78</v>
       </c>
-      <c r="O7" s="13">
+      <c r="O7" s="11">
         <v>0.27</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="10">
         <f t="shared" si="2"/>
         <v>2.7</v>
       </c>
-      <c r="Q7" s="7"/>
+      <c r="Q7" s="5"/>
     </row>
     <row r="8" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37">
+      <c r="A8" s="32">
         <v>6</v>
       </c>
-      <c r="B8" s="126"/>
-      <c r="C8" s="34" t="s">
+      <c r="B8" s="107"/>
+      <c r="C8" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="63" t="s">
+      <c r="D8" s="54" t="s">
         <v>228</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="2" t="s">
         <v>28</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="57" t="s">
+      <c r="H8" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="4">
         <v>2</v>
       </c>
-      <c r="K8" s="17">
+      <c r="K8" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M8" s="13">
+      <c r="M8" s="11">
         <v>0.5</v>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="10">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="O8" s="13">
+      <c r="O8" s="11">
         <v>0.34799999999999998</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="10">
         <f t="shared" si="2"/>
         <v>3.4799999999999995</v>
       </c>
-      <c r="Q8" s="7"/>
-    </row>
-    <row r="9" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="37">
+      <c r="Q8" s="5"/>
+    </row>
+    <row r="9" spans="1:17" s="94" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="32">
         <v>7</v>
       </c>
-      <c r="B9" s="126"/>
-      <c r="C9" s="43" t="s">
+      <c r="B9" s="107"/>
+      <c r="C9" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="64" t="s">
+      <c r="D9" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="44" t="s">
+      <c r="E9" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="F9" s="128" t="s">
+      <c r="F9" s="91" t="s">
         <v>32</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="J9" s="6">
+      <c r="J9" s="4">
         <v>2</v>
       </c>
-      <c r="K9" s="17">
+      <c r="K9" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M9" s="13">
+      <c r="M9" s="11">
         <v>0.97</v>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="10">
         <f t="shared" si="1"/>
         <v>1.94</v>
       </c>
-      <c r="O9" s="13">
+      <c r="O9" s="11">
         <v>0.73899999999999999</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="10">
         <f t="shared" si="2"/>
         <v>7.39</v>
       </c>
-      <c r="Q9" s="7"/>
+      <c r="Q9" s="5"/>
     </row>
     <row r="10" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="37">
+      <c r="A10" s="32">
         <v>8</v>
       </c>
-      <c r="B10" s="126"/>
-      <c r="C10" s="43" t="s">
+      <c r="B10" s="108"/>
+      <c r="C10" s="38" t="s">
         <v>255</v>
       </c>
-      <c r="D10" s="64" t="s">
+      <c r="D10" s="55" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="39" t="s">
         <v>257</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="39" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="127"/>
-      <c r="H10" s="99"/>
-      <c r="I10" s="95" t="s">
-        <v>273</v>
-      </c>
-      <c r="J10" s="98">
+      <c r="G10" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="H10" s="80" t="s">
+        <v>167</v>
+      </c>
+      <c r="I10" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="J10" s="81">
         <v>2</v>
       </c>
-      <c r="K10" s="17">
+      <c r="K10" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L10" s="100"/>
-      <c r="M10" s="101"/>
-      <c r="N10" s="102"/>
-      <c r="O10" s="101"/>
-      <c r="P10" s="102"/>
-      <c r="Q10" s="103"/>
+      <c r="L10" s="138" t="s">
+        <v>145</v>
+      </c>
+      <c r="M10" s="84">
+        <v>0.99</v>
+      </c>
+      <c r="N10" s="10">
+        <f t="shared" si="1"/>
+        <v>1.98</v>
+      </c>
+      <c r="O10" s="84">
+        <v>0.751</v>
+      </c>
+      <c r="P10" s="10">
+        <f t="shared" si="2"/>
+        <v>7.51</v>
+      </c>
+      <c r="Q10" s="86"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="37">
+      <c r="A11" s="32">
         <v>9</v>
       </c>
-      <c r="B11" s="119" t="s">
+      <c r="B11" s="106" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="62" t="s">
+      <c r="D11" s="53" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H11" s="56" t="s">
+      <c r="H11" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="I11" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="16">
         <v>2</v>
       </c>
-      <c r="K11" s="17">
+      <c r="K11" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M11" s="19">
+      <c r="M11" s="17">
         <v>0.67</v>
       </c>
-      <c r="N11" s="20">
+      <c r="N11" s="18">
         <f t="shared" si="1"/>
         <v>1.34</v>
       </c>
-      <c r="O11" s="19">
+      <c r="O11" s="17">
         <v>0.59199999999999997</v>
       </c>
-      <c r="P11" s="20">
+      <c r="P11" s="18">
         <f t="shared" si="2"/>
         <v>5.92</v>
       </c>
-      <c r="Q11" s="21"/>
+      <c r="Q11" s="19"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="37">
+      <c r="A12" s="32">
         <v>10</v>
       </c>
-      <c r="B12" s="120"/>
-      <c r="C12" s="34" t="s">
+      <c r="B12" s="107"/>
+      <c r="C12" s="29" t="s">
         <v>174</v>
       </c>
-      <c r="D12" s="63" t="s">
+      <c r="D12" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="2" t="s">
         <v>40</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H12" s="57" t="s">
+      <c r="H12" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J12" s="4">
         <v>1</v>
       </c>
-      <c r="K12" s="17">
+      <c r="K12" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="11">
         <v>0.27</v>
       </c>
-      <c r="N12" s="12">
+      <c r="N12" s="10">
         <f t="shared" si="1"/>
         <v>0.27</v>
       </c>
-      <c r="O12" s="13">
+      <c r="O12" s="11">
         <v>0.26</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="10">
         <f t="shared" si="2"/>
         <v>1.3</v>
       </c>
-      <c r="Q12" s="7"/>
+      <c r="Q12" s="5"/>
     </row>
     <row r="13" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="37">
+      <c r="A13" s="32">
         <v>11</v>
       </c>
-      <c r="B13" s="120"/>
-      <c r="C13" s="34" t="s">
+      <c r="B13" s="107"/>
+      <c r="C13" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="H13" s="57" t="s">
+      <c r="H13" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="4">
         <v>2</v>
       </c>
-      <c r="K13" s="17">
+      <c r="K13" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="11">
         <v>0.37</v>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="10">
         <f t="shared" si="1"/>
         <v>0.74</v>
       </c>
-      <c r="O13" s="13">
+      <c r="O13" s="11">
         <v>0.29299999999999998</v>
       </c>
-      <c r="P13" s="12">
+      <c r="P13" s="10">
         <f t="shared" si="2"/>
         <v>2.9299999999999997</v>
       </c>
-      <c r="Q13" s="7"/>
+      <c r="Q13" s="5"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="37">
+      <c r="A14" s="32">
         <v>12</v>
       </c>
-      <c r="B14" s="121"/>
-      <c r="C14" s="35" t="s">
+      <c r="B14" s="108"/>
+      <c r="C14" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="56" t="s">
         <v>176</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H14" s="58" t="s">
+      <c r="H14" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I14" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="7">
         <v>1</v>
       </c>
-      <c r="K14" s="17">
+      <c r="K14" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L14" s="22" t="s">
+      <c r="L14" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="M14" s="14">
+      <c r="M14" s="12">
         <v>0.44400000000000001</v>
       </c>
-      <c r="N14" s="23">
+      <c r="N14" s="21">
         <f t="shared" si="1"/>
         <v>0.44400000000000001</v>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="12">
         <v>0.44400000000000001</v>
       </c>
-      <c r="P14" s="23">
+      <c r="P14" s="21">
         <f t="shared" si="2"/>
         <v>2.2200000000000002</v>
       </c>
-      <c r="Q14" s="11"/>
+      <c r="Q14" s="9"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="37">
+      <c r="A15" s="32">
         <v>13</v>
       </c>
-      <c r="B15" s="122" t="s">
+      <c r="B15" s="109" t="s">
         <v>250</v>
       </c>
-      <c r="C15" s="104" t="s">
+      <c r="C15" s="87" t="s">
         <v>238</v>
       </c>
-      <c r="D15" s="62" t="s">
+      <c r="D15" s="53" t="s">
         <v>239</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="H15" s="56" t="s">
+      <c r="H15" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="J15" s="18">
+      <c r="J15" s="16">
         <v>1</v>
       </c>
-      <c r="K15" s="17">
+      <c r="K15" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L15" s="107" t="s">
+      <c r="L15" s="89" t="s">
         <v>226</v>
       </c>
-      <c r="M15" s="19">
+      <c r="M15" s="17">
         <v>0.31</v>
       </c>
-      <c r="N15" s="20">
+      <c r="N15" s="18">
         <f t="shared" si="1"/>
         <v>0.31</v>
       </c>
-      <c r="O15" s="19">
+      <c r="O15" s="17">
         <v>0.31</v>
       </c>
-      <c r="P15" s="20">
+      <c r="P15" s="18">
         <f t="shared" si="2"/>
         <v>1.55</v>
       </c>
-      <c r="Q15" s="21"/>
-    </row>
-    <row r="16" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="37">
+      <c r="Q15" s="19"/>
+    </row>
+    <row r="16" spans="1:17" s="94" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="32">
         <v>14</v>
       </c>
-      <c r="B16" s="123"/>
-      <c r="C16" s="105" t="s">
+      <c r="B16" s="110"/>
+      <c r="C16" s="140" t="s">
         <v>241</v>
       </c>
-      <c r="D16" s="63" t="s">
+      <c r="D16" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="H16" s="57" t="s">
+      <c r="H16" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J16" s="6">
+      <c r="J16" s="4">
         <v>1</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L16" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="M16" s="13">
+      <c r="M16" s="11">
         <v>0.25600000000000001</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="10">
         <f t="shared" si="1"/>
         <v>0.25600000000000001</v>
       </c>
-      <c r="O16" s="13">
+      <c r="O16" s="11">
         <v>0.25600000000000001</v>
       </c>
-      <c r="P16" s="12">
+      <c r="P16" s="10">
         <f t="shared" si="2"/>
         <v>1.28</v>
       </c>
-      <c r="Q16" s="7"/>
+      <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="37">
+      <c r="A17" s="32">
         <v>15</v>
       </c>
-      <c r="B17" s="124"/>
-      <c r="C17" s="106" t="s">
+      <c r="B17" s="111"/>
+      <c r="C17" s="88" t="s">
         <v>244</v>
       </c>
-      <c r="D17" s="129" t="s">
+      <c r="D17" s="92" t="s">
         <v>245</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="G17" s="24" t="s">
+      <c r="G17" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="H17" s="58" t="s">
+      <c r="H17" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I17" s="8" t="s">
+      <c r="I17" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="7">
         <v>1</v>
       </c>
-      <c r="K17" s="10">
+      <c r="K17" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L17" s="22" t="s">
+      <c r="L17" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="M17" s="14">
+      <c r="M17" s="12">
         <v>0.28000000000000003</v>
       </c>
-      <c r="N17" s="23">
+      <c r="N17" s="21">
         <f t="shared" si="1"/>
         <v>0.28000000000000003</v>
       </c>
-      <c r="O17" s="14">
+      <c r="O17" s="12">
         <v>0.28000000000000003</v>
       </c>
-      <c r="P17" s="23">
+      <c r="P17" s="21">
         <f t="shared" si="2"/>
         <v>1.4000000000000001</v>
       </c>
-      <c r="Q17" s="11"/>
+      <c r="Q17" s="9"/>
     </row>
     <row r="18" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="37">
+      <c r="A18" s="32">
         <v>16</v>
       </c>
-      <c r="B18" s="118" t="s">
+      <c r="B18" s="105" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="94" t="s">
+      <c r="C18" s="78" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="54" t="s">
         <v>259</v>
       </c>
-      <c r="E18" s="95" t="s">
+      <c r="E18" s="79" t="s">
         <v>166</v>
       </c>
-      <c r="F18" s="95" t="s">
+      <c r="F18" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="G18" s="96" t="s">
+      <c r="G18" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="H18" s="97" t="s">
+      <c r="H18" s="80" t="s">
         <v>165</v>
       </c>
-      <c r="I18" s="95" t="s">
+      <c r="I18" s="79" t="s">
         <v>132</v>
       </c>
-      <c r="J18" s="98">
+      <c r="J18" s="81">
         <v>2</v>
       </c>
-      <c r="K18" s="99">
+      <c r="K18" s="82">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L18" s="100" t="s">
+      <c r="L18" s="83" t="s">
         <v>145</v>
       </c>
-      <c r="M18" s="101">
+      <c r="M18" s="84">
         <v>2.41</v>
       </c>
-      <c r="N18" s="102">
+      <c r="N18" s="85">
         <f t="shared" si="1"/>
         <v>4.82</v>
       </c>
-      <c r="O18" s="101">
+      <c r="O18" s="84">
         <v>2.41</v>
       </c>
-      <c r="P18" s="102">
+      <c r="P18" s="85">
         <f t="shared" si="2"/>
         <v>24.1</v>
       </c>
-      <c r="Q18" s="103"/>
+      <c r="Q18" s="86"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="37">
+      <c r="A19" s="32">
         <v>17</v>
       </c>
-      <c r="B19" s="116"/>
-      <c r="C19" s="35" t="s">
+      <c r="B19" s="103"/>
+      <c r="C19" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="130" t="s">
+      <c r="D19" s="93" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="24" t="s">
+      <c r="G19" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H19" s="58" t="s">
+      <c r="H19" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I19" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="7">
         <v>1</v>
       </c>
-      <c r="K19" s="17">
+      <c r="K19" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L19" s="22" t="s">
+      <c r="L19" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="M19" s="14">
+      <c r="M19" s="12">
         <v>1.05</v>
       </c>
-      <c r="N19" s="23">
+      <c r="N19" s="21">
         <f t="shared" si="1"/>
         <v>1.05</v>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="12">
         <v>1.05</v>
       </c>
-      <c r="P19" s="23">
+      <c r="P19" s="21">
         <f t="shared" si="2"/>
         <v>5.25</v>
       </c>
-      <c r="Q19" s="11"/>
+      <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="37">
+      <c r="A20" s="32">
         <v>18</v>
       </c>
-      <c r="B20" s="114" t="s">
+      <c r="B20" s="101" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="62" t="s">
+      <c r="D20" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G20" s="26" t="s">
+      <c r="G20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H20" s="56" t="s">
+      <c r="H20" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="I20" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="16">
         <v>2</v>
       </c>
-      <c r="K20" s="17">
+      <c r="K20" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L20" s="16" t="s">
+      <c r="L20" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M20" s="19">
+      <c r="M20" s="17">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N20" s="20">
+      <c r="N20" s="18">
         <f t="shared" si="1"/>
         <v>0.28000000000000003</v>
       </c>
-      <c r="O20" s="19">
+      <c r="O20" s="17">
         <v>0.125</v>
       </c>
-      <c r="P20" s="20">
+      <c r="P20" s="18">
         <f t="shared" si="2"/>
         <v>1.25</v>
       </c>
-      <c r="Q20" s="21"/>
+      <c r="Q20" s="19"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="37">
+      <c r="A21" s="32">
         <v>19</v>
       </c>
-      <c r="B21" s="115"/>
-      <c r="C21" s="34" t="s">
+      <c r="B21" s="102"/>
+      <c r="C21" s="29" t="s">
         <v>181</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="G21" s="45" t="s">
+      <c r="G21" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H21" s="59" t="s">
+      <c r="H21" s="50" t="s">
         <v>165</v>
       </c>
-      <c r="I21" s="44" t="s">
+      <c r="I21" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="J21" s="46">
+      <c r="J21" s="41">
         <v>1</v>
       </c>
-      <c r="K21" s="17">
+      <c r="K21" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L21" s="45" t="s">
+      <c r="L21" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="M21" s="47">
+      <c r="M21" s="42">
         <v>0.5</v>
       </c>
-      <c r="N21" s="48">
+      <c r="N21" s="43">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="O21" s="47">
+      <c r="O21" s="42">
         <v>0.5</v>
       </c>
-      <c r="P21" s="48">
+      <c r="P21" s="43">
         <f t="shared" si="2"/>
         <v>2.5</v>
       </c>
-      <c r="Q21" s="49"/>
+      <c r="Q21" s="44"/>
     </row>
     <row r="22" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="37">
+      <c r="A22" s="32">
         <v>20</v>
       </c>
-      <c r="B22" s="116"/>
-      <c r="C22" s="35" t="s">
+      <c r="B22" s="103"/>
+      <c r="C22" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="65" t="s">
+      <c r="D22" s="56" t="s">
         <v>229</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H22" s="58" t="s">
+      <c r="H22" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I22" s="8" t="s">
+      <c r="I22" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="J22" s="9">
+      <c r="J22" s="7">
         <v>1</v>
       </c>
-      <c r="K22" s="17">
+      <c r="K22" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L22" s="22" t="s">
+      <c r="L22" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="M22" s="14">
+      <c r="M22" s="12">
         <v>0.14000000000000001</v>
       </c>
-      <c r="N22" s="23">
+      <c r="N22" s="21">
         <f t="shared" si="1"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="O22" s="14">
+      <c r="O22" s="12">
         <v>0.14000000000000001</v>
       </c>
-      <c r="P22" s="23">
+      <c r="P22" s="21">
         <f t="shared" si="2"/>
         <v>0.70000000000000007</v>
       </c>
-      <c r="Q22" s="11"/>
-    </row>
-    <row r="23" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="37">
+      <c r="Q22" s="9"/>
+    </row>
+    <row r="23" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="32">
         <v>21</v>
       </c>
-      <c r="B23" s="114" t="s">
+      <c r="B23" s="101" t="s">
         <v>214</v>
       </c>
-      <c r="C23" s="51" t="s">
+      <c r="C23" s="139" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="64" t="s">
+      <c r="D23" s="55" t="s">
         <v>231</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="G23" s="25" t="s">
+      <c r="G23" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H23" s="56" t="s">
+      <c r="H23" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="I23" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="16">
         <v>7</v>
       </c>
-      <c r="K23" s="17">
+      <c r="K23" s="15">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="L23" s="16" t="s">
+      <c r="L23" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M23" s="19">
+      <c r="M23" s="17">
         <v>0.1</v>
       </c>
-      <c r="N23" s="20">
+      <c r="N23" s="18">
         <f t="shared" si="1"/>
         <v>0.70000000000000007</v>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="17">
         <v>5.8000000000000003E-2</v>
       </c>
-      <c r="P23" s="20">
+      <c r="P23" s="18">
         <f t="shared" si="2"/>
         <v>2.0300000000000002</v>
       </c>
-      <c r="Q23" s="21"/>
+      <c r="Q23" s="19"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="37">
+      <c r="A24" s="32">
         <v>22</v>
       </c>
-      <c r="B24" s="115"/>
-      <c r="C24" s="34" t="s">
+      <c r="B24" s="102"/>
+      <c r="C24" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="D24" s="64" t="s">
+      <c r="D24" s="55" t="s">
         <v>185</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="H24" s="57" t="s">
+      <c r="H24" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="4">
         <v>1</v>
       </c>
-      <c r="K24" s="17">
+      <c r="K24" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L24" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M24" s="13">
+      <c r="M24" s="11">
         <v>0.1</v>
       </c>
-      <c r="N24" s="12">
+      <c r="N24" s="10">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O24" s="13">
+      <c r="O24" s="11">
         <v>0.1</v>
       </c>
-      <c r="P24" s="12">
+      <c r="P24" s="10">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q24" s="7"/>
+      <c r="Q24" s="5"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="37">
+      <c r="A25" s="32">
         <v>23</v>
       </c>
-      <c r="B25" s="115"/>
-      <c r="C25" s="34" t="s">
+      <c r="B25" s="102"/>
+      <c r="C25" s="29" t="s">
         <v>184</v>
       </c>
-      <c r="D25" s="64" t="s">
+      <c r="D25" s="55" t="s">
         <v>235</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="H25" s="57" t="s">
+      <c r="H25" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I25" s="44" t="s">
+      <c r="I25" s="39" t="s">
         <v>187</v>
       </c>
-      <c r="J25" s="46">
+      <c r="J25" s="41">
         <v>1</v>
       </c>
-      <c r="K25" s="17">
+      <c r="K25" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L25" s="45" t="s">
+      <c r="L25" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="M25" s="47">
+      <c r="M25" s="42">
         <v>0.1</v>
       </c>
-      <c r="N25" s="48">
+      <c r="N25" s="43">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O25" s="47">
+      <c r="O25" s="42">
         <v>0.1</v>
       </c>
-      <c r="P25" s="48">
+      <c r="P25" s="43">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q25" s="52"/>
+      <c r="Q25" s="45"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="37">
+      <c r="A26" s="32">
         <v>24</v>
       </c>
-      <c r="B26" s="115"/>
-      <c r="C26" s="34" t="s">
+      <c r="B26" s="102"/>
+      <c r="C26" s="29" t="s">
         <v>261</v>
       </c>
-      <c r="D26" s="64" t="s">
+      <c r="D26" s="55" t="s">
         <v>236</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="H26" s="57" t="s">
+      <c r="H26" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I26" s="44" t="s">
+      <c r="I26" s="39" t="s">
         <v>260</v>
       </c>
-      <c r="J26" s="46">
+      <c r="J26" s="41">
         <v>1</v>
       </c>
-      <c r="K26" s="17">
+      <c r="K26" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L26" s="108" t="s">
+      <c r="L26" s="90" t="s">
         <v>226</v>
       </c>
-      <c r="M26" s="47">
+      <c r="M26" s="42">
         <v>0.61</v>
       </c>
-      <c r="N26" s="48">
+      <c r="N26" s="43">
         <f t="shared" si="1"/>
         <v>0.61</v>
       </c>
-      <c r="O26" s="47">
+      <c r="O26" s="42">
         <v>0.61</v>
       </c>
-      <c r="P26" s="48">
+      <c r="P26" s="43">
         <f t="shared" si="2"/>
         <v>3.05</v>
       </c>
-      <c r="Q26" s="52"/>
-    </row>
-    <row r="27" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="37">
+      <c r="Q26" s="45"/>
+    </row>
+    <row r="27" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="32">
         <v>25</v>
       </c>
-      <c r="B27" s="115"/>
-      <c r="C27" s="53" t="s">
+      <c r="B27" s="102"/>
+      <c r="C27" s="46" t="s">
         <v>190</v>
       </c>
-      <c r="D27" s="64" t="s">
+      <c r="D27" s="55" t="s">
         <v>233</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="H27" s="57" t="s">
+      <c r="H27" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="J27" s="6">
+      <c r="J27" s="4">
         <v>3</v>
       </c>
-      <c r="K27" s="17">
+      <c r="K27" s="15">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M27" s="13">
+      <c r="M27" s="11">
         <v>0.1</v>
       </c>
-      <c r="N27" s="12">
+      <c r="N27" s="10">
         <f t="shared" si="1"/>
         <v>0.30000000000000004</v>
       </c>
-      <c r="O27" s="13">
+      <c r="O27" s="11">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="P27" s="12">
+      <c r="P27" s="10">
         <f t="shared" si="2"/>
         <v>0.73499999999999999</v>
       </c>
-      <c r="Q27" s="7"/>
+      <c r="Q27" s="5"/>
     </row>
     <row r="28" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="37">
+      <c r="A28" s="32">
         <v>26</v>
       </c>
-      <c r="B28" s="115"/>
-      <c r="C28" s="34" t="s">
+      <c r="B28" s="102"/>
+      <c r="C28" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="D28" s="64" t="s">
+      <c r="D28" s="55" t="s">
         <v>232</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H28" s="57" t="s">
+      <c r="H28" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="J28" s="6">
+      <c r="J28" s="4">
         <v>1</v>
       </c>
-      <c r="K28" s="17">
+      <c r="K28" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L28" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M28" s="13">
+      <c r="M28" s="11">
         <v>0.13</v>
       </c>
-      <c r="N28" s="12">
+      <c r="N28" s="10">
         <f t="shared" si="1"/>
         <v>0.13</v>
       </c>
-      <c r="O28" s="13">
+      <c r="O28" s="11">
         <v>0.13</v>
       </c>
-      <c r="P28" s="12">
+      <c r="P28" s="10">
         <f t="shared" si="2"/>
         <v>0.65</v>
       </c>
-      <c r="Q28" s="7"/>
-    </row>
-    <row r="29" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="37">
+      <c r="Q28" s="5"/>
+    </row>
+    <row r="29" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="32">
         <v>27</v>
       </c>
-      <c r="B29" s="115"/>
-      <c r="C29" s="53" t="s">
+      <c r="B29" s="102"/>
+      <c r="C29" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="64" t="s">
+      <c r="D29" s="55" t="s">
         <v>234</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="H29" s="57" t="s">
+      <c r="H29" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="4">
         <v>1</v>
       </c>
-      <c r="K29" s="17">
+      <c r="K29" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L29" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M29" s="13">
+      <c r="M29" s="11">
         <v>0.1</v>
       </c>
-      <c r="N29" s="12">
+      <c r="N29" s="10">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O29" s="13">
+      <c r="O29" s="11">
         <v>0.1</v>
       </c>
-      <c r="P29" s="12">
+      <c r="P29" s="10">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q29" s="7"/>
+      <c r="Q29" s="5"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="37">
+      <c r="A30" s="32">
         <v>28</v>
       </c>
-      <c r="B30" s="115"/>
-      <c r="C30" s="34" t="s">
+      <c r="B30" s="102"/>
+      <c r="C30" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="64" t="s">
+      <c r="D30" s="55" t="s">
         <v>230</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="H30" s="57" t="s">
+      <c r="H30" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="4">
         <v>4</v>
       </c>
-      <c r="K30" s="17">
+      <c r="K30" s="15">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="L30" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M30" s="13">
+      <c r="M30" s="11">
         <v>0.24</v>
       </c>
-      <c r="N30" s="12">
+      <c r="N30" s="10">
         <f t="shared" si="1"/>
         <v>0.96</v>
       </c>
-      <c r="O30" s="13">
+      <c r="O30" s="11">
         <v>0.20499999999999999</v>
       </c>
-      <c r="P30" s="12">
+      <c r="P30" s="10">
         <f t="shared" si="2"/>
         <v>4.0999999999999996</v>
       </c>
-      <c r="Q30" s="7"/>
+      <c r="Q30" s="5"/>
     </row>
     <row r="31" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="37">
+      <c r="A31" s="32">
         <v>29</v>
       </c>
-      <c r="B31" s="115"/>
-      <c r="C31" s="34" t="s">
+      <c r="B31" s="102"/>
+      <c r="C31" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="64" t="s">
+      <c r="D31" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="H31" s="57" t="s">
+      <c r="H31" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="J31" s="6">
+      <c r="J31" s="4">
         <v>1</v>
       </c>
-      <c r="K31" s="17">
+      <c r="K31" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L31" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M31" s="13">
+      <c r="M31" s="11">
         <v>0.1</v>
       </c>
-      <c r="N31" s="12">
+      <c r="N31" s="10">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O31" s="13">
+      <c r="O31" s="11">
         <v>0.1</v>
       </c>
-      <c r="P31" s="12">
+      <c r="P31" s="10">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q31" s="7"/>
+      <c r="Q31" s="5"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="37">
+      <c r="A32" s="32">
         <v>30</v>
       </c>
-      <c r="B32" s="115"/>
-      <c r="C32" s="34" t="s">
+      <c r="B32" s="102"/>
+      <c r="C32" s="29" t="s">
         <v>170</v>
       </c>
-      <c r="D32" s="64" t="s">
+      <c r="D32" s="55" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="G32" s="54" t="s">
+      <c r="G32" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H32" s="57" t="s">
+      <c r="H32" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="J32" s="46">
+      <c r="J32" s="41">
         <v>1</v>
       </c>
-      <c r="K32" s="17">
+      <c r="K32" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M32" s="47">
+      <c r="M32" s="42">
         <v>0.92</v>
       </c>
-      <c r="N32" s="48">
+      <c r="N32" s="43">
         <f t="shared" si="1"/>
         <v>0.92</v>
       </c>
-      <c r="O32" s="47">
+      <c r="O32" s="42">
         <v>0.92</v>
       </c>
-      <c r="P32" s="48">
+      <c r="P32" s="43">
         <f t="shared" si="2"/>
         <v>4.6000000000000005</v>
       </c>
-      <c r="Q32" s="52"/>
+      <c r="Q32" s="45"/>
     </row>
     <row r="33" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="37">
+      <c r="A33" s="32">
         <v>31</v>
       </c>
-      <c r="B33" s="115"/>
-      <c r="C33" s="34" t="s">
+      <c r="B33" s="102"/>
+      <c r="C33" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="D33" s="64" t="s">
+      <c r="D33" s="55" t="s">
         <v>77</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G33" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="H33" s="57" t="s">
+      <c r="H33" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I33" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="4">
         <v>1</v>
       </c>
-      <c r="K33" s="17">
+      <c r="K33" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M33" s="13">
+      <c r="M33" s="11">
         <v>0.1</v>
       </c>
-      <c r="N33" s="12">
+      <c r="N33" s="10">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O33" s="13">
+      <c r="O33" s="11">
         <v>0.1</v>
       </c>
-      <c r="P33" s="12">
+      <c r="P33" s="10">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q33" s="7"/>
+      <c r="Q33" s="5"/>
     </row>
     <row r="34" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="37">
+      <c r="A34" s="32">
         <v>32</v>
       </c>
-      <c r="B34" s="115"/>
-      <c r="C34" s="34" t="s">
+      <c r="B34" s="102"/>
+      <c r="C34" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="D34" s="64" t="s">
+      <c r="D34" s="55" t="s">
         <v>80</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="H34" s="57" t="s">
+      <c r="H34" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J34" s="6">
+      <c r="J34" s="4">
         <v>1</v>
       </c>
-      <c r="K34" s="17">
+      <c r="K34" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M34" s="13">
+      <c r="M34" s="11">
         <v>0.1</v>
       </c>
-      <c r="N34" s="12">
+      <c r="N34" s="10">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-      <c r="O34" s="13">
+      <c r="O34" s="11">
         <v>0.1</v>
       </c>
-      <c r="P34" s="12">
+      <c r="P34" s="10">
         <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
-      <c r="Q34" s="7"/>
+      <c r="Q34" s="5"/>
     </row>
     <row r="35" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="37">
+      <c r="A35" s="32">
         <v>33</v>
       </c>
-      <c r="B35" s="115"/>
-      <c r="C35" s="34" t="s">
+      <c r="B35" s="102"/>
+      <c r="C35" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="D35" s="64" t="s">
+      <c r="D35" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="G35" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H35" s="57" t="s">
+      <c r="H35" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I35" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="J35" s="6">
+      <c r="J35" s="4">
         <v>4</v>
       </c>
-      <c r="K35" s="17">
+      <c r="K35" s="15">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M35" s="13">
+      <c r="M35" s="11">
         <v>0.1</v>
       </c>
-      <c r="N35" s="12">
+      <c r="N35" s="10">
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
-      <c r="O35" s="13">
+      <c r="O35" s="11">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="P35" s="12">
+      <c r="P35" s="10">
         <f t="shared" si="2"/>
         <v>0.34</v>
       </c>
-      <c r="Q35" s="7"/>
+      <c r="Q35" s="5"/>
     </row>
     <row r="36" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="37">
+      <c r="A36" s="32">
         <v>34</v>
       </c>
-      <c r="B36" s="61" t="s">
+      <c r="B36" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="36" t="s">
+      <c r="C36" s="31" t="s">
         <v>193</v>
       </c>
-      <c r="D36" s="66" t="s">
+      <c r="D36" s="57" t="s">
         <v>86</v>
       </c>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="22" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F36" s="22" t="s">
         <v>194</v>
       </c>
-      <c r="G36" s="55" t="s">
+      <c r="G36" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="H36" s="60" t="s">
+      <c r="H36" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="I36" s="27" t="s">
+      <c r="I36" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="J36" s="28">
+      <c r="J36" s="23">
         <v>1</v>
       </c>
-      <c r="K36" s="17">
+      <c r="K36" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L36" s="29" t="s">
+      <c r="L36" s="24" t="s">
         <v>145</v>
       </c>
-      <c r="M36" s="30">
+      <c r="M36" s="25">
         <v>0.93</v>
       </c>
-      <c r="N36" s="31">
+      <c r="N36" s="26">
         <f t="shared" si="1"/>
         <v>0.93</v>
       </c>
-      <c r="O36" s="30">
+      <c r="O36" s="25">
         <v>0.93</v>
       </c>
-      <c r="P36" s="31">
+      <c r="P36" s="26">
         <f t="shared" si="2"/>
         <v>4.6500000000000004</v>
       </c>
-      <c r="Q36" s="32"/>
+      <c r="Q36" s="27"/>
     </row>
     <row r="37" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="37">
+      <c r="A37" s="32">
         <v>35</v>
       </c>
-      <c r="B37" s="114" t="s">
+      <c r="B37" s="101" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="84" t="s">
+      <c r="C37" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="62" t="s">
+      <c r="D37" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="E37" s="62" t="s">
+      <c r="E37" s="53" t="s">
         <v>166</v>
       </c>
-      <c r="F37" s="62" t="s">
+      <c r="F37" s="53" t="s">
         <v>90</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="G37" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H37" s="62" t="s">
+      <c r="H37" s="53" t="s">
         <v>165</v>
       </c>
-      <c r="I37" s="62" t="s">
+      <c r="I37" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="J37" s="85">
+      <c r="J37" s="69">
         <v>1</v>
       </c>
-      <c r="K37" s="17">
+      <c r="K37" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L37" s="45" t="s">
+      <c r="L37" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="M37" s="86">
+      <c r="M37" s="70">
         <v>4.3499999999999996</v>
       </c>
-      <c r="N37" s="87">
+      <c r="N37" s="71">
         <f t="shared" si="1"/>
         <v>4.3499999999999996</v>
       </c>
-      <c r="O37" s="86">
+      <c r="O37" s="70">
         <v>4.3499999999999996</v>
       </c>
-      <c r="P37" s="87">
+      <c r="P37" s="71">
         <f t="shared" si="2"/>
         <v>21.75</v>
       </c>
-      <c r="Q37" s="88"/>
+      <c r="Q37" s="72"/>
     </row>
     <row r="38" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="37">
+      <c r="A38" s="32">
         <v>36</v>
       </c>
-      <c r="B38" s="115"/>
-      <c r="C38" s="43" t="s">
+      <c r="B38" s="102"/>
+      <c r="C38" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="D38" s="64" t="s">
+      <c r="D38" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="E38" s="44" t="s">
+      <c r="E38" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="F38" s="44" t="s">
+      <c r="F38" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="G38" s="50" t="s">
+      <c r="G38" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H38" s="57" t="s">
+      <c r="H38" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I38" s="44" t="s">
+      <c r="I38" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="J38" s="46">
+      <c r="J38" s="41">
         <v>1</v>
       </c>
-      <c r="K38" s="17">
+      <c r="K38" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L38" s="45" t="s">
+      <c r="L38" s="40" t="s">
         <v>172</v>
       </c>
-      <c r="M38" s="47">
+      <c r="M38" s="42">
         <v>3.71</v>
       </c>
-      <c r="N38" s="48">
+      <c r="N38" s="43">
         <f t="shared" si="1"/>
         <v>3.71</v>
       </c>
-      <c r="O38" s="47">
+      <c r="O38" s="42">
         <v>3.71</v>
       </c>
-      <c r="P38" s="48">
+      <c r="P38" s="43">
         <f t="shared" si="2"/>
         <v>18.55</v>
       </c>
-      <c r="Q38" s="49"/>
+      <c r="Q38" s="44"/>
     </row>
     <row r="39" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="37">
+      <c r="A39" s="32">
         <v>37</v>
       </c>
-      <c r="B39" s="115"/>
-      <c r="C39" s="34" t="s">
+      <c r="B39" s="102"/>
+      <c r="C39" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="D39" s="63" t="s">
+      <c r="D39" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="G39" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="H39" s="57" t="s">
+      <c r="H39" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I39" s="4" t="s">
+      <c r="I39" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J39" s="6">
+      <c r="J39" s="4">
         <v>1</v>
       </c>
-      <c r="K39" s="17">
+      <c r="K39" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L39" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M39" s="13">
+      <c r="M39" s="11">
         <v>0.99</v>
       </c>
-      <c r="N39" s="12">
+      <c r="N39" s="10">
         <f t="shared" si="1"/>
         <v>0.99</v>
       </c>
-      <c r="O39" s="13">
+      <c r="O39" s="11">
         <v>0.99</v>
       </c>
-      <c r="P39" s="12">
+      <c r="P39" s="10">
         <f t="shared" si="2"/>
         <v>4.95</v>
       </c>
-      <c r="Q39" s="7"/>
+      <c r="Q39" s="5"/>
     </row>
     <row r="40" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="37">
+      <c r="A40" s="32">
         <v>38</v>
       </c>
-      <c r="B40" s="115"/>
-      <c r="C40" s="34" t="s">
+      <c r="B40" s="102"/>
+      <c r="C40" s="29" t="s">
         <v>197</v>
       </c>
-      <c r="D40" s="63" t="s">
+      <c r="D40" s="54" t="s">
         <v>99</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="G40" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="H40" s="57" t="s">
+      <c r="H40" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I40" s="4"/>
-      <c r="J40" s="6">
+      <c r="I40" s="2"/>
+      <c r="J40" s="4">
         <v>1</v>
       </c>
-      <c r="K40" s="17">
+      <c r="K40" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L40" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M40" s="13">
+      <c r="M40" s="11">
         <v>3.9</v>
       </c>
-      <c r="N40" s="12">
+      <c r="N40" s="10">
         <f t="shared" si="1"/>
         <v>3.9</v>
       </c>
-      <c r="O40" s="13">
+      <c r="O40" s="11">
         <v>3.9</v>
       </c>
-      <c r="P40" s="12">
+      <c r="P40" s="10">
         <f t="shared" si="2"/>
         <v>19.5</v>
       </c>
-      <c r="Q40" s="7"/>
+      <c r="Q40" s="5"/>
     </row>
     <row r="41" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="37">
+      <c r="A41" s="32">
         <v>39</v>
       </c>
-      <c r="B41" s="115"/>
-      <c r="C41" s="43" t="s">
+      <c r="B41" s="102"/>
+      <c r="C41" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="D41" s="64" t="s">
+      <c r="D41" s="55" t="s">
         <v>102</v>
       </c>
-      <c r="E41" s="93" t="s">
+      <c r="E41" s="77" t="s">
         <v>166</v>
       </c>
-      <c r="F41" s="44" t="s">
+      <c r="F41" s="39" t="s">
         <v>103</v>
       </c>
-      <c r="G41" s="50" t="s">
+      <c r="G41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H41" s="57" t="s">
+      <c r="H41" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I41" s="44" t="s">
+      <c r="I41" s="39" t="s">
         <v>162</v>
       </c>
-      <c r="J41" s="46">
+      <c r="J41" s="41">
         <v>1</v>
       </c>
-      <c r="K41" s="17">
+      <c r="K41" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L41" s="45" t="s">
+      <c r="L41" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="M41" s="47">
+      <c r="M41" s="42">
         <v>0.46600000000000003</v>
       </c>
-      <c r="N41" s="48">
+      <c r="N41" s="43">
         <f t="shared" si="1"/>
         <v>0.46600000000000003</v>
       </c>
-      <c r="O41" s="47">
+      <c r="O41" s="42">
         <v>0.46600000000000003</v>
       </c>
-      <c r="P41" s="48">
+      <c r="P41" s="43">
         <f t="shared" si="2"/>
         <v>2.33</v>
       </c>
-      <c r="Q41" s="49"/>
+      <c r="Q41" s="44"/>
     </row>
     <row r="42" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="37">
+      <c r="A42" s="32">
         <v>40</v>
       </c>
-      <c r="B42" s="115"/>
-      <c r="C42" s="34" t="s">
+      <c r="B42" s="102"/>
+      <c r="C42" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="64" t="s">
+      <c r="D42" s="55" t="s">
         <v>237</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F42" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G42" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H42" s="57" t="s">
+      <c r="H42" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I42" s="4" t="s">
+      <c r="I42" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J42" s="6">
+      <c r="J42" s="4">
         <v>3</v>
       </c>
-      <c r="K42" s="17">
+      <c r="K42" s="15">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="L42" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M42" s="13">
+      <c r="M42" s="11">
         <v>0.52</v>
       </c>
-      <c r="N42" s="12">
+      <c r="N42" s="10">
         <f t="shared" si="1"/>
         <v>1.56</v>
       </c>
-      <c r="O42" s="13">
+      <c r="O42" s="11">
         <v>0.42299999999999999</v>
       </c>
-      <c r="P42" s="12">
+      <c r="P42" s="10">
         <f t="shared" si="2"/>
         <v>6.3449999999999998</v>
       </c>
-      <c r="Q42" s="7"/>
+      <c r="Q42" s="5"/>
     </row>
     <row r="43" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="37">
+      <c r="A43" s="32">
         <v>41</v>
       </c>
-      <c r="B43" s="115"/>
-      <c r="C43" s="34" t="s">
+      <c r="B43" s="102"/>
+      <c r="C43" s="29" t="s">
         <v>201</v>
       </c>
-      <c r="D43" s="64" t="s">
+      <c r="D43" s="55" t="s">
         <v>202</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F43" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G43" s="45" t="s">
+      <c r="G43" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="H43" s="57" t="s">
+      <c r="H43" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I43" s="44"/>
-      <c r="J43" s="46">
+      <c r="I43" s="39"/>
+      <c r="J43" s="41">
         <v>1</v>
       </c>
-      <c r="K43" s="17">
+      <c r="K43" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L43" s="45" t="s">
+      <c r="L43" s="40" t="s">
         <v>145</v>
       </c>
-      <c r="M43" s="47">
+      <c r="M43" s="42">
         <v>0.57999999999999996</v>
       </c>
-      <c r="N43" s="48">
+      <c r="N43" s="43">
         <f t="shared" si="1"/>
         <v>0.57999999999999996</v>
       </c>
-      <c r="O43" s="47">
+      <c r="O43" s="42">
         <v>0.57999999999999996</v>
       </c>
-      <c r="P43" s="48">
+      <c r="P43" s="43">
         <f t="shared" si="2"/>
         <v>2.9</v>
       </c>
-      <c r="Q43" s="49"/>
+      <c r="Q43" s="44"/>
     </row>
     <row r="44" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="37">
+      <c r="A44" s="32">
         <v>42</v>
       </c>
-      <c r="B44" s="115"/>
-      <c r="C44" s="34" t="s">
+      <c r="B44" s="102"/>
+      <c r="C44" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="D44" s="64" t="s">
+      <c r="D44" s="55" t="s">
         <v>206</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F44" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="G44" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H44" s="57" t="s">
+      <c r="H44" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I44" s="4"/>
-      <c r="J44" s="6">
+      <c r="I44" s="2"/>
+      <c r="J44" s="4">
         <v>1</v>
       </c>
-      <c r="K44" s="17">
+      <c r="K44" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M44" s="13">
+      <c r="M44" s="11">
         <v>0.48</v>
       </c>
-      <c r="N44" s="12">
+      <c r="N44" s="10">
         <f t="shared" si="1"/>
         <v>0.48</v>
       </c>
-      <c r="O44" s="13">
+      <c r="O44" s="11">
         <v>0.48</v>
       </c>
-      <c r="P44" s="12">
+      <c r="P44" s="10">
         <f t="shared" si="2"/>
         <v>2.4</v>
       </c>
-      <c r="Q44" s="7"/>
+      <c r="Q44" s="5"/>
     </row>
     <row r="45" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="37">
+      <c r="A45" s="32">
         <v>43</v>
       </c>
-      <c r="B45" s="116"/>
-      <c r="C45" s="34" t="s">
+      <c r="B45" s="103"/>
+      <c r="C45" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="D45" s="65" t="s">
+      <c r="D45" s="56" t="s">
         <v>109</v>
       </c>
-      <c r="E45" s="8" t="s">
+      <c r="E45" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F45" s="8" t="s">
+      <c r="F45" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="G45" s="24" t="s">
+      <c r="G45" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H45" s="58" t="s">
+      <c r="H45" s="49" t="s">
         <v>165</v>
       </c>
-      <c r="I45" s="8" t="s">
+      <c r="I45" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="J45" s="9">
+      <c r="J45" s="7">
         <v>1</v>
       </c>
-      <c r="K45" s="17">
+      <c r="K45" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L45" s="22" t="s">
+      <c r="L45" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="M45" s="14">
+      <c r="M45" s="12">
         <v>7.32</v>
       </c>
-      <c r="N45" s="23">
+      <c r="N45" s="21">
         <f t="shared" si="1"/>
         <v>7.32</v>
       </c>
-      <c r="O45" s="14">
+      <c r="O45" s="12">
         <v>7.32</v>
       </c>
-      <c r="P45" s="23">
+      <c r="P45" s="21">
         <f t="shared" si="2"/>
         <v>36.6</v>
       </c>
-      <c r="Q45" s="11"/>
+      <c r="Q45" s="9"/>
     </row>
     <row r="46" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="37">
+      <c r="A46" s="32">
         <v>44</v>
       </c>
-      <c r="B46" s="114" t="s">
+      <c r="B46" s="101" t="s">
         <v>111</v>
       </c>
-      <c r="C46" s="33" t="s">
+      <c r="C46" s="28" t="s">
         <v>211</v>
       </c>
-      <c r="D46" s="62" t="s">
+      <c r="D46" s="53" t="s">
         <v>253</v>
       </c>
-      <c r="E46" s="15" t="s">
+      <c r="E46" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="F46" s="15" t="s">
+      <c r="F46" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="G46" s="16" t="s">
+      <c r="G46" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H46" s="56" t="s">
+      <c r="H46" s="47" t="s">
         <v>165</v>
       </c>
-      <c r="I46" s="15" t="s">
+      <c r="I46" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="J46" s="18">
+      <c r="J46" s="16">
         <v>7</v>
       </c>
-      <c r="K46" s="17">
+      <c r="K46" s="15">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="L46" s="16" t="s">
+      <c r="L46" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="M46" s="19">
+      <c r="M46" s="17">
         <v>0.15</v>
       </c>
-      <c r="N46" s="20">
+      <c r="N46" s="18">
         <f t="shared" si="1"/>
         <v>1.05</v>
       </c>
-      <c r="O46" s="19">
+      <c r="O46" s="17">
         <v>0.14099999999999999</v>
       </c>
-      <c r="P46" s="20">
+      <c r="P46" s="18">
         <f t="shared" si="2"/>
         <v>4.9349999999999996</v>
       </c>
-      <c r="Q46" s="21"/>
+      <c r="Q46" s="19"/>
     </row>
     <row r="47" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="37">
+      <c r="A47" s="32">
         <v>45</v>
       </c>
-      <c r="B47" s="115"/>
-      <c r="C47" s="34" t="s">
+      <c r="B47" s="102"/>
+      <c r="C47" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="D47" s="63" t="s">
+      <c r="D47" s="54" t="s">
         <v>252</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F47" s="4" t="s">
+      <c r="F47" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="G47" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H47" s="57" t="s">
+      <c r="H47" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I47" s="4" t="s">
+      <c r="I47" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J47" s="6">
+      <c r="J47" s="4">
         <v>2</v>
       </c>
-      <c r="K47" s="17">
+      <c r="K47" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="L47" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M47" s="13">
+      <c r="M47" s="11">
         <v>0.21</v>
       </c>
-      <c r="N47" s="12">
+      <c r="N47" s="10">
         <f t="shared" si="1"/>
         <v>0.42</v>
       </c>
-      <c r="O47" s="13">
+      <c r="O47" s="11">
         <v>0.19400000000000001</v>
       </c>
-      <c r="P47" s="12">
+      <c r="P47" s="10">
         <f t="shared" si="2"/>
         <v>1.94</v>
       </c>
-      <c r="Q47" s="7"/>
+      <c r="Q47" s="5"/>
     </row>
     <row r="48" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="37">
+      <c r="A48" s="32">
         <v>46</v>
       </c>
-      <c r="B48" s="115"/>
-      <c r="C48" s="34" t="s">
+      <c r="B48" s="102"/>
+      <c r="C48" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="D48" s="63" t="s">
+      <c r="D48" s="54" t="s">
         <v>212</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="E48" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F48" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G48" s="1" t="s">
+      <c r="G48" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H48" s="57" t="s">
+      <c r="H48" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I48" s="4" t="s">
+      <c r="I48" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J48" s="6">
+      <c r="J48" s="4">
         <v>5</v>
       </c>
-      <c r="K48" s="17">
+      <c r="K48" s="15">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="L48" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="M48" s="13">
+      <c r="M48" s="11">
         <v>0.13300000000000001</v>
       </c>
-      <c r="N48" s="12">
+      <c r="N48" s="10">
         <f t="shared" si="1"/>
         <v>0.66500000000000004</v>
       </c>
-      <c r="O48" s="13">
+      <c r="O48" s="11">
         <v>0.13300000000000001</v>
       </c>
-      <c r="P48" s="12">
+      <c r="P48" s="10">
         <f t="shared" si="2"/>
         <v>3.3250000000000002</v>
       </c>
-      <c r="Q48" s="7"/>
+      <c r="Q48" s="5"/>
     </row>
     <row r="49" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="37">
+      <c r="A49" s="32">
         <v>47</v>
       </c>
-      <c r="B49" s="115"/>
-      <c r="C49" s="34" t="s">
+      <c r="B49" s="102"/>
+      <c r="C49" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="D49" s="63" t="s">
+      <c r="D49" s="54" t="s">
         <v>251</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="E49" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="F49" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G49" s="1" t="s">
+      <c r="G49" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H49" s="57" t="s">
+      <c r="H49" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I49" s="4" t="s">
+      <c r="I49" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J49" s="6">
+      <c r="J49" s="4">
         <v>3</v>
       </c>
-      <c r="K49" s="17">
+      <c r="K49" s="15">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="L49" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M49" s="13">
+      <c r="M49" s="11">
         <v>0.33</v>
       </c>
-      <c r="N49" s="12">
+      <c r="N49" s="10">
         <f t="shared" si="1"/>
         <v>0.99</v>
       </c>
-      <c r="O49" s="13">
+      <c r="O49" s="11">
         <v>0.308</v>
       </c>
-      <c r="P49" s="12">
+      <c r="P49" s="10">
         <f t="shared" si="2"/>
         <v>4.62</v>
       </c>
-      <c r="Q49" s="7"/>
+      <c r="Q49" s="5"/>
     </row>
     <row r="50" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="37">
+      <c r="A50" s="32">
         <v>48</v>
       </c>
-      <c r="B50" s="115"/>
-      <c r="C50" s="34" t="s">
+      <c r="B50" s="102"/>
+      <c r="C50" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="D50" s="63" t="s">
+      <c r="D50" s="54" t="s">
         <v>121</v>
       </c>
-      <c r="E50" s="4" t="s">
+      <c r="E50" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F50" s="2" t="s">
         <v>122</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H50" s="57" t="s">
+      <c r="H50" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="I50" s="4" t="s">
+      <c r="I50" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="J50" s="6">
+      <c r="J50" s="4">
         <v>1</v>
       </c>
-      <c r="K50" s="17">
+      <c r="K50" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="L50" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="M50" s="13">
+      <c r="M50" s="11">
         <v>3</v>
       </c>
-      <c r="N50" s="12">
+      <c r="N50" s="10">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="O50" s="13">
+      <c r="O50" s="11">
         <v>3</v>
       </c>
-      <c r="P50" s="12">
+      <c r="P50" s="10">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="Q50" s="7"/>
+      <c r="Q50" s="5"/>
     </row>
     <row r="51" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="37">
+      <c r="A51" s="32">
         <v>49</v>
       </c>
-      <c r="B51" s="117"/>
-      <c r="C51" s="83" t="s">
+      <c r="B51" s="104"/>
+      <c r="C51" s="67" t="s">
         <v>216</v>
       </c>
-      <c r="D51" s="77" t="s">
+      <c r="D51" s="61" t="s">
         <v>217</v>
       </c>
-      <c r="E51" s="77" t="s">
+      <c r="E51" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="F51" s="78" t="s">
+      <c r="F51" s="62" t="s">
         <v>218</v>
       </c>
-      <c r="G51" s="79" t="s">
+      <c r="G51" s="63" t="s">
         <v>167</v>
       </c>
-      <c r="H51" s="79" t="s">
+      <c r="H51" s="63" t="s">
         <v>167</v>
       </c>
-      <c r="I51" s="79" t="s">
+      <c r="I51" s="63" t="s">
         <v>267</v>
       </c>
-      <c r="J51" s="80">
+      <c r="J51" s="64">
         <v>1</v>
       </c>
-      <c r="K51" s="17">
+      <c r="K51" s="15">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L51" s="79" t="s">
+      <c r="L51" s="63" t="s">
         <v>167</v>
       </c>
-      <c r="M51" s="81" t="s">
+      <c r="M51" s="65" t="s">
         <v>167</v>
       </c>
-      <c r="N51" s="81" t="s">
+      <c r="N51" s="65" t="s">
         <v>167</v>
       </c>
-      <c r="O51" s="81" t="s">
+      <c r="O51" s="65" t="s">
         <v>167</v>
       </c>
-      <c r="P51" s="81" t="s">
+      <c r="P51" s="65" t="s">
         <v>167</v>
       </c>
-      <c r="Q51" s="82" t="s">
+      <c r="Q51" s="66" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="52" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="37">
+      <c r="A52" s="32">
         <v>50</v>
       </c>
-      <c r="B52" s="116"/>
-      <c r="C52" s="70" t="s">
+      <c r="B52" s="104"/>
+      <c r="C52" s="112" t="s">
         <v>124</v>
       </c>
-      <c r="D52" s="71" t="s">
+      <c r="D52" s="113" t="s">
         <v>125</v>
       </c>
-      <c r="E52" s="71" t="s">
+      <c r="E52" s="113" t="s">
         <v>166</v>
       </c>
-      <c r="F52" s="72" t="s">
+      <c r="F52" s="114" t="s">
         <v>144</v>
       </c>
-      <c r="G52" s="73" t="s">
+      <c r="G52" s="115" t="s">
         <v>167</v>
       </c>
-      <c r="H52" s="73" t="s">
+      <c r="H52" s="115" t="s">
         <v>167</v>
       </c>
-      <c r="I52" s="73" t="s">
+      <c r="I52" s="115" t="s">
         <v>267</v>
       </c>
-      <c r="J52" s="74">
+      <c r="J52" s="116">
         <v>4</v>
       </c>
-      <c r="K52" s="17">
+      <c r="K52" s="117">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L52" s="73" t="s">
+      <c r="L52" s="115" t="s">
         <v>167</v>
       </c>
-      <c r="M52" s="75" t="s">
+      <c r="M52" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="N52" s="75" t="s">
+      <c r="N52" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="O52" s="75" t="s">
+      <c r="O52" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="P52" s="75" t="s">
+      <c r="P52" s="118" t="s">
         <v>167</v>
       </c>
-      <c r="Q52" s="76" t="s">
+      <c r="Q52" s="119" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="53" spans="1:17" s="131" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="37">
+    <row r="53" spans="1:17" s="94" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="32">
         <v>51</v>
       </c>
-      <c r="B53" s="136" t="s">
+      <c r="B53" s="106" t="s">
         <v>263</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C53" s="28" t="s">
         <v>265</v>
       </c>
-      <c r="E53" s="4" t="s">
+      <c r="D53" s="126"/>
+      <c r="E53" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="F53" s="4" t="s">
+      <c r="F53" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="G53" s="132" t="s">
+      <c r="G53" s="127" t="s">
         <v>266</v>
       </c>
-      <c r="H53" s="132" t="s">
+      <c r="H53" s="127" t="s">
         <v>266</v>
       </c>
-      <c r="I53" s="132" t="s">
+      <c r="I53" s="127" t="s">
         <v>268</v>
       </c>
-      <c r="J53" s="134">
+      <c r="J53" s="128">
         <v>2</v>
       </c>
-      <c r="K53" s="135">
+      <c r="K53" s="129">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L53" s="133" t="s">
-        <v>270</v>
-      </c>
-      <c r="M53" s="132"/>
-      <c r="N53" s="132"/>
-      <c r="O53" s="132"/>
-      <c r="P53" s="132"/>
-      <c r="Q53" s="132"/>
+      <c r="L53" s="130"/>
+      <c r="M53" s="127"/>
+      <c r="N53" s="127"/>
+      <c r="O53" s="127"/>
+      <c r="P53" s="127"/>
+      <c r="Q53" s="131"/>
     </row>
     <row r="54" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="37">
+      <c r="A54" s="32">
         <v>52</v>
       </c>
-      <c r="B54" s="137"/>
-      <c r="C54" s="138" t="s">
-        <v>274</v>
-      </c>
-      <c r="E54" s="4" t="s">
+      <c r="B54" s="107"/>
+      <c r="C54" s="95" t="s">
+        <v>273</v>
+      </c>
+      <c r="D54" s="121"/>
+      <c r="E54" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="F54" s="4" t="s">
+      <c r="F54" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="G54" s="140" t="s">
+      <c r="G54" s="122" t="s">
         <v>266</v>
       </c>
-      <c r="H54" s="140" t="s">
+      <c r="H54" s="122" t="s">
         <v>266</v>
       </c>
-      <c r="J54" s="134">
+      <c r="I54" s="121"/>
+      <c r="J54" s="123">
         <v>2</v>
       </c>
-      <c r="K54" s="135">
+      <c r="K54" s="124">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L54" s="139" t="s">
+      <c r="L54" s="73"/>
+      <c r="M54" s="121"/>
+      <c r="N54" s="121"/>
+      <c r="O54" s="121"/>
+      <c r="P54" s="121"/>
+      <c r="Q54" s="132"/>
+    </row>
+    <row r="55" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="32">
+        <v>53</v>
+      </c>
+      <c r="B55" s="107"/>
+      <c r="C55" s="125"/>
+      <c r="D55" s="121"/>
+      <c r="E55" s="121"/>
+      <c r="F55" s="123" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="55" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="37">
-        <v>53</v>
-      </c>
-      <c r="B55" s="137"/>
-      <c r="F55" s="134" t="s">
-        <v>271</v>
-      </c>
-      <c r="J55" s="134">
+      <c r="G55" s="122" t="s">
+        <v>266</v>
+      </c>
+      <c r="H55" s="122" t="s">
+        <v>266</v>
+      </c>
+      <c r="I55" s="121"/>
+      <c r="J55" s="123">
         <v>1</v>
       </c>
-      <c r="K55" s="135">
+      <c r="K55" s="124">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A56" s="37">
+      <c r="L55" s="121"/>
+      <c r="M55" s="121"/>
+      <c r="N55" s="121"/>
+      <c r="O55" s="121"/>
+      <c r="P55" s="121"/>
+      <c r="Q55" s="132"/>
+    </row>
+    <row r="56" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="120">
         <v>54</v>
       </c>
-      <c r="B56" s="137"/>
-      <c r="F56" s="134" t="s">
-        <v>272</v>
-      </c>
-      <c r="J56" s="134">
+      <c r="B56" s="108"/>
+      <c r="C56" s="133"/>
+      <c r="D56" s="134"/>
+      <c r="E56" s="134"/>
+      <c r="F56" s="135" t="s">
+        <v>271</v>
+      </c>
+      <c r="G56" s="122" t="s">
+        <v>266</v>
+      </c>
+      <c r="H56" s="122" t="s">
+        <v>266</v>
+      </c>
+      <c r="I56" s="134"/>
+      <c r="J56" s="135">
         <v>1</v>
       </c>
-      <c r="K56" s="135">
+      <c r="K56" s="136">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
+      <c r="L56" s="134"/>
+      <c r="M56" s="134"/>
+      <c r="N56" s="134"/>
+      <c r="O56" s="134"/>
+      <c r="P56" s="134"/>
+      <c r="Q56" s="137"/>
     </row>
     <row r="57" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J57" s="112" t="s">
+      <c r="J57" s="99" t="s">
         <v>163</v>
       </c>
-      <c r="K57" s="112"/>
-      <c r="L57" s="112"/>
-      <c r="M57" s="112"/>
-      <c r="N57" s="38"/>
-      <c r="O57" s="39"/>
-      <c r="P57" s="40">
-        <f>SUM(P3:P50)</f>
-        <v>243.95400000000001</v>
+      <c r="K57" s="99"/>
+      <c r="L57" s="99"/>
+      <c r="M57" s="99"/>
+      <c r="N57" s="33"/>
+      <c r="O57" s="34"/>
+      <c r="P57" s="35">
+        <f>SUM(P3:P56)</f>
+        <v>251.46400000000003</v>
       </c>
     </row>
     <row r="58" spans="1:17" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="J58" s="113" t="s">
+      <c r="J58" s="100" t="s">
         <v>164</v>
       </c>
-      <c r="K58" s="113"/>
-      <c r="L58" s="113"/>
-      <c r="M58" s="113"/>
-      <c r="N58" s="41">
-        <f>SUM(N3:N50)</f>
-        <v>52.83100000000001</v>
-      </c>
-      <c r="O58" s="42"/>
-      <c r="P58" s="41">
+      <c r="K58" s="100"/>
+      <c r="L58" s="100"/>
+      <c r="M58" s="100"/>
+      <c r="N58" s="36">
+        <f>SUM(N11:N57)</f>
+        <v>45.460999999999991</v>
+      </c>
+      <c r="O58" s="37"/>
+      <c r="P58" s="36">
         <f>P57/5</f>
-        <v>48.790800000000004</v>
+        <v>50.292800000000007</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="J57:M57"/>
     <mergeCell ref="J58:M58"/>
@@ -5080,6 +5136,8 @@
     <mergeCell ref="B23:B35"/>
     <mergeCell ref="B11:B14"/>
     <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="B3:B10"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <conditionalFormatting sqref="N58">
@@ -5270,11 +5328,10 @@
     <hyperlink ref="L15" r:id="rId77"/>
     <hyperlink ref="L26" r:id="rId78"/>
     <hyperlink ref="G26" r:id="rId79" display="https://lcsc.com/brand-detail/396.html"/>
-    <hyperlink ref="L54" r:id="rId80"/>
-    <hyperlink ref="L53" r:id="rId81"/>
+    <hyperlink ref="L10" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId82"/>
+  <pageSetup orientation="portrait" r:id="rId81"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
#71 . Formatting adjusted in designs.
</commit_message>
<xml_diff>
--- a/Documents/Deliverables/BOM/Digikey_BOM.xlsx
+++ b/Documents/Deliverables/BOM/Digikey_BOM.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\FranciscoGimenez-HCDSHardware\Documents\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9666C967-82A3-4C5A-A546-06CDD849E73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,6 +25,7 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -815,15 +817,9 @@
     <t>ESP32-WROOM-32E(4MB)</t>
   </si>
   <si>
-    <t>U7, U8, U19, U10</t>
-  </si>
-  <si>
     <t>P1, P2, P3, P4, P5, P6</t>
   </si>
   <si>
-    <t>J3, J24, J25, J28, J29</t>
-  </si>
-  <si>
     <t>LED4, LED5</t>
   </si>
   <si>
@@ -870,9 +866,6 @@
   </si>
   <si>
     <t>3 POS 2.54mm female header</t>
-  </si>
-  <si>
-    <t>J10, J11, J12, J13, J20, J30</t>
   </si>
   <si>
     <t>HDR_F_1X3</t>
@@ -895,12 +888,21 @@
   <si>
     <t xml:space="preserve">801-47-003-10-001000
 </t>
+  </si>
+  <si>
+    <t>U7, U8, U19, U10,U11</t>
+  </si>
+  <si>
+    <t>J3, J24, J25, J28, J29, J31</t>
+  </si>
+  <si>
+    <t>J10, J11, J12, J13, J17,  J20, J30</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1831,51 +1833,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2020,6 +1977,51 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2301,7 +2303,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2325,90 +2327,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="172" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="115"/>
-      <c r="C1" s="115"/>
-      <c r="D1" s="115"/>
-      <c r="E1" s="115"/>
-      <c r="F1" s="115"/>
-      <c r="G1" s="115"/>
-      <c r="H1" s="115"/>
-      <c r="I1" s="115"/>
-      <c r="J1" s="115"/>
-      <c r="K1" s="115"/>
-      <c r="L1" s="115"/>
-      <c r="M1" s="115"/>
-      <c r="N1" s="115"/>
-      <c r="O1" s="115"/>
-      <c r="P1" s="115"/>
-      <c r="Q1" s="116"/>
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
+      <c r="I1" s="173"/>
+      <c r="J1" s="173"/>
+      <c r="K1" s="173"/>
+      <c r="L1" s="173"/>
+      <c r="M1" s="173"/>
+      <c r="N1" s="173"/>
+      <c r="O1" s="173"/>
+      <c r="P1" s="173"/>
+      <c r="Q1" s="174"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="173" t="s">
+      <c r="B2" s="158" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="173" t="s">
+      <c r="C2" s="158" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="173" t="s">
+      <c r="D2" s="158" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="173" t="s">
+      <c r="E2" s="158" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="173" t="s">
+      <c r="F2" s="158" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="173" t="s">
+      <c r="G2" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="173" t="s">
+      <c r="H2" s="158" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="173" t="s">
+      <c r="I2" s="158" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="173" t="s">
+      <c r="J2" s="158" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="173" t="s">
+      <c r="K2" s="158" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="173" t="s">
+      <c r="L2" s="158" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="173" t="s">
+      <c r="M2" s="158" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="173" t="s">
+      <c r="N2" s="158" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="173" t="s">
+      <c r="O2" s="158" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="173" t="s">
+      <c r="P2" s="158" t="s">
         <v>130</v>
       </c>
-      <c r="Q2" s="173" t="s">
+      <c r="Q2" s="158" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="172">
+      <c r="A3" s="157">
         <v>1</v>
       </c>
-      <c r="B3" s="119" t="s">
+      <c r="B3" s="163" t="s">
         <v>190</v>
       </c>
       <c r="C3" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="166" t="s">
+      <c r="D3" s="151" t="s">
         <v>196</v>
       </c>
       <c r="E3" s="13" t="s">
@@ -2433,10 +2435,10 @@
         <f>J3*5</f>
         <v>65</v>
       </c>
-      <c r="L3" s="133" t="s">
+      <c r="L3" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="M3" s="137">
+      <c r="M3" s="122">
         <v>0.1</v>
       </c>
       <c r="N3" s="17">
@@ -2453,14 +2455,14 @@
       <c r="Q3" s="18"/>
     </row>
     <row r="4" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="172">
+      <c r="A4" s="157">
         <v>2</v>
       </c>
-      <c r="B4" s="120"/>
+      <c r="B4" s="164"/>
       <c r="C4" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="167" t="s">
+      <c r="D4" s="152" t="s">
         <v>254</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -2505,10 +2507,10 @@
       <c r="Q4" s="5"/>
     </row>
     <row r="5" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="172">
+      <c r="A5" s="157">
         <v>3</v>
       </c>
-      <c r="B5" s="120"/>
+      <c r="B5" s="164"/>
       <c r="C5" s="21" t="s">
         <v>197</v>
       </c>
@@ -2557,10 +2559,10 @@
       <c r="Q5" s="5"/>
     </row>
     <row r="6" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="172">
+      <c r="A6" s="157">
         <v>4</v>
       </c>
-      <c r="B6" s="120"/>
+      <c r="B6" s="164"/>
       <c r="C6" s="21" t="s">
         <v>21</v>
       </c>
@@ -2589,7 +2591,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="L6" s="174" t="s">
+      <c r="L6" s="159" t="s">
         <v>129</v>
       </c>
       <c r="M6" s="11">
@@ -2609,10 +2611,10 @@
       <c r="Q6" s="5"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="172">
+      <c r="A7" s="157">
         <v>5</v>
       </c>
-      <c r="B7" s="120"/>
+      <c r="B7" s="164"/>
       <c r="C7" s="21" t="s">
         <v>24</v>
       </c>
@@ -2661,10 +2663,10 @@
       <c r="Q7" s="5"/>
     </row>
     <row r="8" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="172">
+      <c r="A8" s="157">
         <v>6</v>
       </c>
-      <c r="B8" s="120"/>
+      <c r="B8" s="164"/>
       <c r="C8" s="28" t="s">
         <v>28</v>
       </c>
@@ -2713,10 +2715,10 @@
       <c r="Q8" s="5"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="172">
+      <c r="A9" s="157">
         <v>7</v>
       </c>
-      <c r="B9" s="120"/>
+      <c r="B9" s="164"/>
       <c r="C9" s="21" t="s">
         <v>255</v>
       </c>
@@ -2745,7 +2747,7 @@
         <f>J9*5</f>
         <v>10</v>
       </c>
-      <c r="L9" s="174" t="s">
+      <c r="L9" s="159" t="s">
         <v>149</v>
       </c>
       <c r="M9" s="11">
@@ -2765,14 +2767,14 @@
       <c r="Q9" s="104"/>
     </row>
     <row r="10" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="172">
+      <c r="A10" s="157">
         <v>8</v>
       </c>
-      <c r="B10" s="121"/>
+      <c r="B10" s="165"/>
       <c r="C10" s="107" t="s">
         <v>226</v>
       </c>
-      <c r="D10" s="168" t="s">
+      <c r="D10" s="153" t="s">
         <v>227</v>
       </c>
       <c r="E10" s="108" t="s">
@@ -2793,11 +2795,11 @@
       <c r="J10" s="111">
         <v>2</v>
       </c>
-      <c r="K10" s="129">
+      <c r="K10" s="114">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L10" s="152" t="s">
+      <c r="L10" s="137" t="s">
         <v>129</v>
       </c>
       <c r="M10" s="112">
@@ -2817,16 +2819,16 @@
       <c r="Q10" s="113"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="172">
+      <c r="A11" s="157">
         <v>9</v>
       </c>
-      <c r="B11" s="124" t="s">
+      <c r="B11" s="168" t="s">
         <v>31</v>
       </c>
       <c r="C11" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="138" t="s">
+      <c r="D11" s="123" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="58" t="s">
@@ -2851,7 +2853,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L11" s="130" t="s">
+      <c r="L11" s="115" t="s">
         <v>129</v>
       </c>
       <c r="M11" s="102">
@@ -2871,10 +2873,10 @@
       <c r="Q11" s="64"/>
     </row>
     <row r="12" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="172">
+      <c r="A12" s="157">
         <v>10</v>
       </c>
-      <c r="B12" s="124"/>
+      <c r="B12" s="168"/>
       <c r="C12" s="21" t="s">
         <v>154</v>
       </c>
@@ -2923,14 +2925,14 @@
       <c r="Q12" s="5"/>
     </row>
     <row r="13" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="172">
+      <c r="A13" s="157">
         <v>11</v>
       </c>
-      <c r="B13" s="124"/>
+      <c r="B13" s="168"/>
       <c r="C13" s="82" t="s">
         <v>155</v>
       </c>
-      <c r="D13" s="170" t="s">
+      <c r="D13" s="155" t="s">
         <v>156</v>
       </c>
       <c r="E13" s="83" t="s">
@@ -2955,7 +2957,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L13" s="132" t="s">
+      <c r="L13" s="117" t="s">
         <v>159</v>
       </c>
       <c r="M13" s="62">
@@ -2975,16 +2977,16 @@
       <c r="Q13" s="88"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="172">
+      <c r="A14" s="157">
         <v>12</v>
       </c>
-      <c r="B14" s="126" t="s">
+      <c r="B14" s="175" t="s">
         <v>223</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="D14" s="169" t="s">
+      <c r="D14" s="154" t="s">
         <v>212</v>
       </c>
       <c r="E14" s="13" t="s">
@@ -3009,10 +3011,10 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L14" s="133" t="s">
+      <c r="L14" s="118" t="s">
         <v>201</v>
       </c>
-      <c r="M14" s="137">
+      <c r="M14" s="122">
         <v>0.31</v>
       </c>
       <c r="N14" s="17">
@@ -3029,10 +3031,10 @@
       <c r="Q14" s="18"/>
     </row>
     <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="172">
+      <c r="A15" s="157">
         <v>13</v>
       </c>
-      <c r="B15" s="127"/>
+      <c r="B15" s="176"/>
       <c r="C15" s="66" t="s">
         <v>214</v>
       </c>
@@ -3081,10 +3083,10 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="172">
+      <c r="A16" s="157">
         <v>14</v>
       </c>
-      <c r="B16" s="127"/>
+      <c r="B16" s="176"/>
       <c r="C16" s="21" t="s">
         <v>217</v>
       </c>
@@ -3133,15 +3135,15 @@
       <c r="Q16" s="5"/>
     </row>
     <row r="17" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="172">
+      <c r="A17" s="157">
         <v>15</v>
       </c>
-      <c r="B17" s="128"/>
-      <c r="C17" s="134" t="s">
+      <c r="B17" s="177"/>
+      <c r="C17" s="119" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="171" t="s">
-        <v>262</v>
+      <c r="D17" s="156" t="s">
+        <v>260</v>
       </c>
       <c r="E17" s="110" t="s">
         <v>41</v>
@@ -3161,40 +3163,40 @@
       <c r="J17" s="111">
         <v>2</v>
       </c>
-      <c r="K17" s="129">
+      <c r="K17" s="114">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L17" s="135" t="s">
+      <c r="L17" s="120" t="s">
         <v>129</v>
       </c>
       <c r="M17" s="62">
         <v>0.37</v>
       </c>
-      <c r="N17" s="131">
+      <c r="N17" s="116">
         <f t="shared" si="1"/>
         <v>0.74</v>
       </c>
       <c r="O17" s="112">
         <v>0.29299999999999998</v>
       </c>
-      <c r="P17" s="131">
+      <c r="P17" s="116">
         <f t="shared" si="2"/>
         <v>2.9299999999999997</v>
       </c>
       <c r="Q17" s="113"/>
     </row>
     <row r="18" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="172">
+      <c r="A18" s="157">
         <v>16</v>
       </c>
-      <c r="B18" s="119" t="s">
+      <c r="B18" s="163" t="s">
         <v>43</v>
       </c>
       <c r="C18" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="169" t="s">
+      <c r="D18" s="154" t="s">
         <v>230</v>
       </c>
       <c r="E18" s="13" t="s">
@@ -3219,10 +3221,10 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L18" s="133" t="s">
+      <c r="L18" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="M18" s="137">
+      <c r="M18" s="122">
         <v>2.4900000000000002</v>
       </c>
       <c r="N18" s="17">
@@ -3239,14 +3241,14 @@
       <c r="Q18" s="18"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="172">
+      <c r="A19" s="157">
         <v>17</v>
       </c>
-      <c r="B19" s="121"/>
+      <c r="B19" s="165"/>
       <c r="C19" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="171" t="s">
+      <c r="D19" s="156" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="6" t="s">
@@ -3271,7 +3273,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L19" s="176" t="s">
+      <c r="L19" s="161" t="s">
         <v>159</v>
       </c>
       <c r="M19" s="12">
@@ -3291,16 +3293,16 @@
       <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="172">
+      <c r="A20" s="157">
         <v>18</v>
       </c>
-      <c r="B20" s="124" t="s">
+      <c r="B20" s="168" t="s">
         <v>49</v>
       </c>
       <c r="C20" s="96" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="144" t="s">
+      <c r="D20" s="129" t="s">
         <v>51</v>
       </c>
       <c r="E20" s="98" t="s">
@@ -3325,7 +3327,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L20" s="147" t="s">
+      <c r="L20" s="132" t="s">
         <v>129</v>
       </c>
       <c r="M20" s="102">
@@ -3345,10 +3347,10 @@
       <c r="Q20" s="104"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="172">
+      <c r="A21" s="157">
         <v>19</v>
       </c>
-      <c r="B21" s="124"/>
+      <c r="B21" s="168"/>
       <c r="C21" s="21" t="s">
         <v>53</v>
       </c>
@@ -3397,14 +3399,14 @@
       <c r="Q21" s="5"/>
     </row>
     <row r="22" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="172">
+      <c r="A22" s="157">
         <v>20</v>
       </c>
-      <c r="B22" s="124"/>
+      <c r="B22" s="168"/>
       <c r="C22" s="96" t="s">
         <v>161</v>
       </c>
-      <c r="D22" s="144" t="s">
+      <c r="D22" s="129" t="s">
         <v>54</v>
       </c>
       <c r="E22" s="98" t="s">
@@ -3416,49 +3418,49 @@
       <c r="G22" s="98" t="s">
         <v>56</v>
       </c>
-      <c r="H22" s="144" t="s">
+      <c r="H22" s="129" t="s">
         <v>145</v>
       </c>
-      <c r="I22" s="145" t="s">
+      <c r="I22" s="130" t="s">
         <v>142</v>
       </c>
-      <c r="J22" s="146">
+      <c r="J22" s="131">
         <v>1</v>
       </c>
       <c r="K22" s="101">
         <f>J22*5</f>
         <v>5</v>
       </c>
-      <c r="L22" s="147" t="s">
+      <c r="L22" s="132" t="s">
         <v>129</v>
       </c>
       <c r="M22" s="62">
         <v>0.5</v>
       </c>
-      <c r="N22" s="149">
+      <c r="N22" s="134">
         <f>M22*J22</f>
         <v>0.5</v>
       </c>
-      <c r="O22" s="148">
+      <c r="O22" s="133">
         <v>0.5</v>
       </c>
-      <c r="P22" s="149">
+      <c r="P22" s="134">
         <f>O22*K22</f>
         <v>2.5</v>
       </c>
       <c r="Q22" s="104"/>
     </row>
     <row r="23" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="172">
+      <c r="A23" s="157">
         <v>21</v>
       </c>
-      <c r="B23" s="119" t="s">
+      <c r="B23" s="163" t="s">
         <v>191</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="169" t="s">
+      <c r="D23" s="154" t="s">
         <v>205</v>
       </c>
       <c r="E23" s="13" t="s">
@@ -3473,20 +3475,20 @@
       <c r="H23" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="I23" s="136" t="s">
+      <c r="I23" s="121" t="s">
         <v>122</v>
       </c>
-      <c r="J23" s="150">
+      <c r="J23" s="135">
         <v>4</v>
       </c>
       <c r="K23" s="14">
         <f t="shared" ref="K23:K35" si="3">J23*5</f>
         <v>20</v>
       </c>
-      <c r="L23" s="133" t="s">
+      <c r="L23" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="M23" s="137">
+      <c r="M23" s="122">
         <v>0.3</v>
       </c>
       <c r="N23" s="17">
@@ -3503,15 +3505,15 @@
       <c r="Q23" s="18"/>
     </row>
     <row r="24" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="172">
+      <c r="A24" s="157">
         <v>22</v>
       </c>
-      <c r="B24" s="120"/>
+      <c r="B24" s="164"/>
       <c r="C24" s="21" t="s">
         <v>63</v>
       </c>
       <c r="D24" s="38" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>58</v>
@@ -3520,7 +3522,7 @@
         <v>64</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H24" s="36" t="s">
         <v>145</v>
@@ -3528,7 +3530,7 @@
       <c r="I24" s="83" t="s">
         <v>120</v>
       </c>
-      <c r="J24" s="143">
+      <c r="J24" s="128">
         <v>1</v>
       </c>
       <c r="K24" s="61">
@@ -3555,10 +3557,10 @@
       <c r="Q24" s="5"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="172">
+      <c r="A25" s="157">
         <v>23</v>
       </c>
-      <c r="B25" s="120"/>
+      <c r="B25" s="164"/>
       <c r="C25" s="21" t="s">
         <v>57</v>
       </c>
@@ -3572,7 +3574,7 @@
         <v>59</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H25" s="36" t="s">
         <v>145</v>
@@ -3580,7 +3582,7 @@
       <c r="I25" s="83" t="s">
         <v>118</v>
       </c>
-      <c r="J25" s="143">
+      <c r="J25" s="128">
         <v>7</v>
       </c>
       <c r="K25" s="61">
@@ -3607,10 +3609,10 @@
       <c r="Q25" s="34"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="172">
+      <c r="A26" s="157">
         <v>24</v>
       </c>
-      <c r="B26" s="120"/>
+      <c r="B26" s="164"/>
       <c r="C26" s="21" t="s">
         <v>69</v>
       </c>
@@ -3632,7 +3634,7 @@
       <c r="I26" s="83" t="s">
         <v>123</v>
       </c>
-      <c r="J26" s="143">
+      <c r="J26" s="128">
         <v>1</v>
       </c>
       <c r="K26" s="61">
@@ -3659,10 +3661,10 @@
       <c r="Q26" s="34"/>
     </row>
     <row r="27" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="172">
+      <c r="A27" s="157">
         <v>25</v>
       </c>
-      <c r="B27" s="120"/>
+      <c r="B27" s="164"/>
       <c r="C27" s="21" t="s">
         <v>169</v>
       </c>
@@ -3684,7 +3686,7 @@
       <c r="I27" s="83" t="s">
         <v>171</v>
       </c>
-      <c r="J27" s="143">
+      <c r="J27" s="128">
         <v>3</v>
       </c>
       <c r="K27" s="61">
@@ -3711,10 +3713,10 @@
       <c r="Q27" s="5"/>
     </row>
     <row r="28" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="172">
+      <c r="A28" s="157">
         <v>26</v>
       </c>
-      <c r="B28" s="120"/>
+      <c r="B28" s="164"/>
       <c r="C28" s="21" t="s">
         <v>65</v>
       </c>
@@ -3728,7 +3730,7 @@
         <v>66</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H28" s="36" t="s">
         <v>145</v>
@@ -3736,7 +3738,7 @@
       <c r="I28" s="83" t="s">
         <v>121</v>
       </c>
-      <c r="J28" s="143">
+      <c r="J28" s="128">
         <v>1</v>
       </c>
       <c r="K28" s="61">
@@ -3763,10 +3765,10 @@
       <c r="Q28" s="5"/>
     </row>
     <row r="29" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="172">
+      <c r="A29" s="157">
         <v>27</v>
       </c>
-      <c r="B29" s="120"/>
+      <c r="B29" s="164"/>
       <c r="C29" s="21" t="s">
         <v>60</v>
       </c>
@@ -3788,7 +3790,7 @@
       <c r="I29" s="83" t="s">
         <v>119</v>
       </c>
-      <c r="J29" s="143">
+      <c r="J29" s="128">
         <v>1</v>
       </c>
       <c r="K29" s="61">
@@ -3815,10 +3817,10 @@
       <c r="Q29" s="5"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="172">
+      <c r="A30" s="157">
         <v>28</v>
       </c>
-      <c r="B30" s="120"/>
+      <c r="B30" s="164"/>
       <c r="C30" s="21" t="s">
         <v>164</v>
       </c>
@@ -3840,7 +3842,7 @@
       <c r="I30" s="83" t="s">
         <v>167</v>
       </c>
-      <c r="J30" s="143">
+      <c r="J30" s="128">
         <v>1</v>
       </c>
       <c r="K30" s="61">
@@ -3867,10 +3869,10 @@
       <c r="Q30" s="5"/>
     </row>
     <row r="31" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="172">
+      <c r="A31" s="157">
         <v>29</v>
       </c>
-      <c r="B31" s="120"/>
+      <c r="B31" s="164"/>
       <c r="C31" s="21" t="s">
         <v>232</v>
       </c>
@@ -3892,7 +3894,7 @@
       <c r="I31" s="83" t="s">
         <v>231</v>
       </c>
-      <c r="J31" s="143">
+      <c r="J31" s="128">
         <v>1</v>
       </c>
       <c r="K31" s="61">
@@ -3919,10 +3921,10 @@
       <c r="Q31" s="5"/>
     </row>
     <row r="32" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="172">
+      <c r="A32" s="157">
         <v>30</v>
       </c>
-      <c r="B32" s="120"/>
+      <c r="B32" s="164"/>
       <c r="C32" s="21" t="s">
         <v>150</v>
       </c>
@@ -3944,7 +3946,7 @@
       <c r="I32" s="83" t="s">
         <v>124</v>
       </c>
-      <c r="J32" s="143">
+      <c r="J32" s="128">
         <v>1</v>
       </c>
       <c r="K32" s="61">
@@ -3971,10 +3973,10 @@
       <c r="Q32" s="34"/>
     </row>
     <row r="33" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="172">
+      <c r="A33" s="157">
         <v>31</v>
       </c>
-      <c r="B33" s="120"/>
+      <c r="B33" s="164"/>
       <c r="C33" s="21" t="s">
         <v>72</v>
       </c>
@@ -3988,7 +3990,7 @@
         <v>74</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H33" s="36" t="s">
         <v>145</v>
@@ -3996,7 +3998,7 @@
       <c r="I33" s="83" t="s">
         <v>125</v>
       </c>
-      <c r="J33" s="143">
+      <c r="J33" s="128">
         <v>1</v>
       </c>
       <c r="K33" s="61">
@@ -4023,12 +4025,12 @@
       <c r="Q33" s="5"/>
     </row>
     <row r="34" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="172">
+      <c r="A34" s="157">
         <v>32</v>
       </c>
-      <c r="B34" s="120"/>
+      <c r="B34" s="164"/>
       <c r="C34" s="21" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D34" s="38" t="s">
         <v>75</v>
@@ -4048,7 +4050,7 @@
       <c r="I34" s="83" t="s">
         <v>126</v>
       </c>
-      <c r="J34" s="143">
+      <c r="J34" s="128">
         <v>1</v>
       </c>
       <c r="K34" s="61">
@@ -4075,14 +4077,14 @@
       <c r="Q34" s="5"/>
     </row>
     <row r="35" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="172">
+      <c r="A35" s="157">
         <v>33</v>
       </c>
-      <c r="B35" s="121"/>
+      <c r="B35" s="165"/>
       <c r="C35" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D35" s="168" t="s">
+      <c r="D35" s="153" t="s">
         <v>78</v>
       </c>
       <c r="E35" s="6" t="s">
@@ -4092,7 +4094,7 @@
         <v>79</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H35" s="37" t="s">
         <v>145</v>
@@ -4100,14 +4102,14 @@
       <c r="I35" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="J35" s="151">
+      <c r="J35" s="136">
         <v>4</v>
       </c>
-      <c r="K35" s="129">
+      <c r="K35" s="114">
         <f t="shared" si="3"/>
         <v>20</v>
       </c>
-      <c r="L35" s="152" t="s">
+      <c r="L35" s="137" t="s">
         <v>129</v>
       </c>
       <c r="M35" s="62">
@@ -4127,7 +4129,7 @@
       <c r="Q35" s="9"/>
     </row>
     <row r="36" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="172">
+      <c r="A36" s="157">
         <v>34</v>
       </c>
       <c r="B36" s="78" t="s">
@@ -4161,7 +4163,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L36" s="147" t="s">
+      <c r="L36" s="132" t="s">
         <v>129</v>
       </c>
       <c r="M36" s="16">
@@ -4181,10 +4183,10 @@
       <c r="Q36" s="104"/>
     </row>
     <row r="37" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="172">
+      <c r="A37" s="157">
         <v>35</v>
       </c>
-      <c r="B37" s="119" t="s">
+      <c r="B37" s="163" t="s">
         <v>82</v>
       </c>
       <c r="C37" s="50" t="s">
@@ -4215,10 +4217,10 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L37" s="133" t="s">
+      <c r="L37" s="118" t="s">
         <v>129</v>
       </c>
-      <c r="M37" s="137">
+      <c r="M37" s="122">
         <v>4.4379</v>
       </c>
       <c r="N37" s="53">
@@ -4235,10 +4237,10 @@
       <c r="Q37" s="54"/>
     </row>
     <row r="38" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="172">
+      <c r="A38" s="157">
         <v>36</v>
       </c>
-      <c r="B38" s="123"/>
+      <c r="B38" s="166"/>
       <c r="C38" s="21" t="s">
         <v>90</v>
       </c>
@@ -4284,13 +4286,13 @@
         <f>O38*K38</f>
         <v>5.15</v>
       </c>
-      <c r="Q38" s="153"/>
+      <c r="Q38" s="138"/>
     </row>
     <row r="39" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="172">
+      <c r="A39" s="157">
         <v>37</v>
       </c>
-      <c r="B39" s="120"/>
+      <c r="B39" s="164"/>
       <c r="C39" s="28" t="s">
         <v>86</v>
       </c>
@@ -4339,10 +4341,10 @@
       <c r="Q39" s="33"/>
     </row>
     <row r="40" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="172">
+      <c r="A40" s="157">
         <v>38</v>
       </c>
-      <c r="B40" s="120"/>
+      <c r="B40" s="164"/>
       <c r="C40" s="21" t="s">
         <v>176</v>
       </c>
@@ -4389,10 +4391,10 @@
       <c r="Q40" s="5"/>
     </row>
     <row r="41" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="172">
+      <c r="A41" s="157">
         <v>39</v>
       </c>
-      <c r="B41" s="120"/>
+      <c r="B41" s="164"/>
       <c r="C41" s="28" t="s">
         <v>95</v>
       </c>
@@ -4441,15 +4443,15 @@
       <c r="Q41" s="33"/>
     </row>
     <row r="42" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="172">
+      <c r="A42" s="157">
         <v>40</v>
       </c>
-      <c r="B42" s="120"/>
+      <c r="B42" s="164"/>
       <c r="C42" s="82" t="s">
         <v>99</v>
       </c>
-      <c r="D42" s="154" t="s">
-        <v>259</v>
+      <c r="D42" s="139" t="s">
+        <v>282</v>
       </c>
       <c r="E42" s="83" t="s">
         <v>100</v>
@@ -4467,13 +4469,13 @@
         <v>142</v>
       </c>
       <c r="J42" s="85">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K42" s="3">
         <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="L42" s="132" t="s">
+        <v>25</v>
+      </c>
+      <c r="L42" s="117" t="s">
         <v>129</v>
       </c>
       <c r="M42" s="11">
@@ -4481,22 +4483,22 @@
       </c>
       <c r="N42" s="87">
         <f t="shared" si="1"/>
-        <v>2.08</v>
+        <v>2.6</v>
       </c>
       <c r="O42" s="86">
-        <v>0.42299999999999999</v>
+        <v>0.3876</v>
       </c>
       <c r="P42" s="87">
         <f t="shared" si="2"/>
-        <v>8.4599999999999991</v>
+        <v>9.69</v>
       </c>
       <c r="Q42" s="88"/>
     </row>
     <row r="43" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="172">
+      <c r="A43" s="157">
         <v>41</v>
       </c>
-      <c r="B43" s="120"/>
+      <c r="B43" s="164"/>
       <c r="C43" s="21" t="s">
         <v>184</v>
       </c>
@@ -4545,14 +4547,14 @@
       <c r="Q43" s="5"/>
     </row>
     <row r="44" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="172">
+      <c r="A44" s="157">
         <v>42</v>
       </c>
-      <c r="B44" s="120"/>
+      <c r="B44" s="164"/>
       <c r="C44" s="57" t="s">
         <v>180</v>
       </c>
-      <c r="D44" s="155" t="s">
+      <c r="D44" s="140" t="s">
         <v>181</v>
       </c>
       <c r="E44" s="58" t="s">
@@ -4567,38 +4569,38 @@
       <c r="H44" s="59" t="s">
         <v>145</v>
       </c>
-      <c r="I44" s="139"/>
-      <c r="J44" s="140">
+      <c r="I44" s="124"/>
+      <c r="J44" s="125">
         <v>1</v>
       </c>
       <c r="K44" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L44" s="130" t="s">
+      <c r="L44" s="115" t="s">
         <v>129</v>
       </c>
       <c r="M44" s="11">
         <v>0.57999999999999996</v>
       </c>
-      <c r="N44" s="142">
+      <c r="N44" s="127">
         <f t="shared" si="1"/>
         <v>0.57999999999999996</v>
       </c>
-      <c r="O44" s="141">
+      <c r="O44" s="126">
         <v>0.57999999999999996</v>
       </c>
-      <c r="P44" s="142">
+      <c r="P44" s="127">
         <f t="shared" si="2"/>
         <v>2.9</v>
       </c>
-      <c r="Q44" s="156"/>
+      <c r="Q44" s="141"/>
     </row>
     <row r="45" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="172">
+      <c r="A45" s="157">
         <v>43</v>
       </c>
-      <c r="B45" s="121"/>
+      <c r="B45" s="165"/>
       <c r="C45" s="22" t="s">
         <v>184</v>
       </c>
@@ -4621,11 +4623,11 @@
       <c r="J45" s="7">
         <v>1</v>
       </c>
-      <c r="K45" s="129">
+      <c r="K45" s="114">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L45" s="152" t="s">
+      <c r="L45" s="137" t="s">
         <v>129</v>
       </c>
       <c r="M45" s="62">
@@ -4645,26 +4647,26 @@
       <c r="Q45" s="9"/>
     </row>
     <row r="46" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="172">
+      <c r="A46" s="157">
         <v>44</v>
       </c>
-      <c r="B46" s="119" t="s">
+      <c r="B46" s="163" t="s">
         <v>105</v>
       </c>
-      <c r="C46" s="162" t="s">
-        <v>270</v>
+      <c r="C46" s="147" t="s">
+        <v>268</v>
       </c>
       <c r="D46" s="105" t="s">
         <v>224</v>
       </c>
-      <c r="E46" s="163" t="s">
-        <v>271</v>
-      </c>
-      <c r="F46" s="164" t="s">
-        <v>281</v>
-      </c>
-      <c r="G46" s="136" t="s">
-        <v>280</v>
+      <c r="E46" s="148" t="s">
+        <v>269</v>
+      </c>
+      <c r="F46" s="149" t="s">
+        <v>278</v>
+      </c>
+      <c r="G46" s="121" t="s">
+        <v>277</v>
       </c>
       <c r="H46" s="36" t="s">
         <v>145</v>
@@ -4672,17 +4674,17 @@
       <c r="I46" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="J46" s="150">
+      <c r="J46" s="135">
         <v>3</v>
       </c>
       <c r="K46" s="67">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="L46" s="175" t="s">
+      <c r="L46" s="160" t="s">
         <v>129</v>
       </c>
-      <c r="M46" s="137">
+      <c r="M46" s="122">
         <v>1.35</v>
       </c>
       <c r="N46" s="17">
@@ -4699,24 +4701,24 @@
       <c r="Q46" s="18"/>
     </row>
     <row r="47" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="172">
+      <c r="A47" s="157">
         <v>45</v>
       </c>
-      <c r="B47" s="120"/>
+      <c r="B47" s="164"/>
       <c r="C47" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="D47" s="41" t="s">
+        <v>271</v>
+      </c>
+      <c r="E47" s="56" t="s">
         <v>272</v>
       </c>
-      <c r="D47" s="41" t="s">
-        <v>273</v>
-      </c>
-      <c r="E47" s="56" t="s">
-        <v>274</v>
-      </c>
       <c r="F47" s="29" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H47" s="36" t="s">
         <v>145</v>
@@ -4724,14 +4726,14 @@
       <c r="I47" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J47" s="143">
+      <c r="J47" s="128">
         <v>2</v>
       </c>
       <c r="K47" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L47" s="174" t="s">
+      <c r="L47" s="159" t="s">
         <v>129</v>
       </c>
       <c r="M47" s="11">
@@ -4751,24 +4753,24 @@
       <c r="Q47" s="5"/>
     </row>
     <row r="48" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="172">
+      <c r="A48" s="157">
         <v>46</v>
       </c>
-      <c r="B48" s="120"/>
+      <c r="B48" s="164"/>
       <c r="C48" s="28" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D48" s="41" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="E48" s="56" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F48" s="29" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H48" s="36" t="s">
         <v>145</v>
@@ -4776,14 +4778,14 @@
       <c r="I48" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J48" s="143">
-        <v>5</v>
+      <c r="J48" s="128">
+        <v>6</v>
       </c>
       <c r="K48" s="3">
         <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="L48" s="174" t="s">
+        <v>30</v>
+      </c>
+      <c r="L48" s="159" t="s">
         <v>129</v>
       </c>
       <c r="M48" s="11">
@@ -4791,36 +4793,36 @@
       </c>
       <c r="N48" s="10">
         <f t="shared" si="1"/>
-        <v>3.15</v>
+        <v>3.7800000000000002</v>
       </c>
       <c r="O48" s="11">
         <v>0.63</v>
       </c>
       <c r="P48" s="10">
         <f t="shared" si="2"/>
-        <v>15.75</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="Q48" s="5"/>
     </row>
     <row r="49" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="172">
+      <c r="A49" s="157">
         <v>47</v>
       </c>
-      <c r="B49" s="120"/>
+      <c r="B49" s="164"/>
       <c r="C49" s="28" t="s">
+        <v>275</v>
+      </c>
+      <c r="D49" s="41" t="s">
+        <v>284</v>
+      </c>
+      <c r="E49" s="56" t="s">
+        <v>276</v>
+      </c>
+      <c r="F49" s="29" t="s">
+        <v>281</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>277</v>
-      </c>
-      <c r="D49" s="41" t="s">
-        <v>278</v>
-      </c>
-      <c r="E49" s="56" t="s">
-        <v>279</v>
-      </c>
-      <c r="F49" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="H49" s="36" t="s">
         <v>145</v>
@@ -4828,14 +4830,14 @@
       <c r="I49" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J49" s="143">
-        <v>6</v>
+      <c r="J49" s="128">
+        <v>7</v>
       </c>
       <c r="K49" s="3">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="L49" s="174" t="s">
+        <v>35</v>
+      </c>
+      <c r="L49" s="159" t="s">
         <v>129</v>
       </c>
       <c r="M49" s="11">
@@ -4843,22 +4845,22 @@
       </c>
       <c r="N49" s="10">
         <f t="shared" si="1"/>
-        <v>6.12</v>
+        <v>7.1400000000000006</v>
       </c>
       <c r="O49" s="11">
         <v>1.02</v>
       </c>
       <c r="P49" s="10">
         <f t="shared" si="2"/>
-        <v>30.6</v>
+        <v>35.700000000000003</v>
       </c>
       <c r="Q49" s="5"/>
     </row>
     <row r="50" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="172">
+      <c r="A50" s="157">
         <v>48</v>
       </c>
-      <c r="B50" s="120"/>
+      <c r="B50" s="164"/>
       <c r="C50" s="21" t="s">
         <v>106</v>
       </c>
@@ -4887,7 +4889,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L50" s="130" t="s">
+      <c r="L50" s="115" t="s">
         <v>129</v>
       </c>
       <c r="M50" s="62">
@@ -4907,10 +4909,10 @@
       <c r="Q50" s="5"/>
     </row>
     <row r="51" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="172">
+      <c r="A51" s="157">
         <v>49</v>
       </c>
-      <c r="B51" s="122"/>
+      <c r="B51" s="167"/>
       <c r="C51" s="49" t="s">
         <v>193</v>
       </c>
@@ -4959,15 +4961,15 @@
       </c>
     </row>
     <row r="52" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="172">
+      <c r="A52" s="157">
         <v>50</v>
       </c>
-      <c r="B52" s="121"/>
+      <c r="B52" s="165"/>
       <c r="C52" s="89" t="s">
         <v>110</v>
       </c>
-      <c r="D52" s="165" t="s">
-        <v>260</v>
+      <c r="D52" s="150" t="s">
+        <v>259</v>
       </c>
       <c r="E52" s="90" t="s">
         <v>146</v>
@@ -4987,11 +4989,11 @@
       <c r="J52" s="93">
         <v>4</v>
       </c>
-      <c r="K52" s="129">
+      <c r="K52" s="114">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L52" s="152" t="s">
+      <c r="L52" s="137" t="s">
         <v>147</v>
       </c>
       <c r="M52" s="94" t="s">
@@ -5011,52 +5013,52 @@
       </c>
     </row>
     <row r="53" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="172">
+      <c r="A53" s="157">
         <v>51</v>
       </c>
-      <c r="B53" s="124" t="s">
+      <c r="B53" s="168" t="s">
         <v>234</v>
       </c>
       <c r="C53" s="57" t="s">
         <v>236</v>
       </c>
-      <c r="D53" s="157"/>
+      <c r="D53" s="142"/>
       <c r="E53" s="58" t="s">
         <v>146</v>
       </c>
       <c r="F53" s="58" t="s">
         <v>235</v>
       </c>
-      <c r="G53" s="158" t="s">
+      <c r="G53" s="143" t="s">
         <v>237</v>
       </c>
-      <c r="H53" s="158" t="s">
+      <c r="H53" s="143" t="s">
         <v>237</v>
       </c>
-      <c r="I53" s="158" t="s">
+      <c r="I53" s="143" t="s">
         <v>239</v>
       </c>
-      <c r="J53" s="159">
+      <c r="J53" s="144">
         <v>2</v>
       </c>
-      <c r="K53" s="160">
+      <c r="K53" s="145">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L53" s="130" t="s">
+      <c r="L53" s="115" t="s">
         <v>246</v>
       </c>
-      <c r="M53" s="158"/>
-      <c r="N53" s="158"/>
-      <c r="O53" s="158"/>
-      <c r="P53" s="158"/>
-      <c r="Q53" s="161"/>
+      <c r="M53" s="143"/>
+      <c r="N53" s="143"/>
+      <c r="O53" s="143"/>
+      <c r="P53" s="143"/>
+      <c r="Q53" s="146"/>
     </row>
     <row r="54" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="172">
+      <c r="A54" s="157">
         <v>52</v>
       </c>
-      <c r="B54" s="124"/>
+      <c r="B54" s="168"/>
       <c r="C54" s="66" t="s">
         <v>244</v>
       </c>
@@ -5091,10 +5093,10 @@
       <c r="Q54" s="73"/>
     </row>
     <row r="55" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="172">
+      <c r="A55" s="157">
         <v>53</v>
       </c>
-      <c r="B55" s="124"/>
+      <c r="B55" s="168"/>
       <c r="C55" s="79" t="s">
         <v>247</v>
       </c>
@@ -5125,10 +5127,10 @@
       <c r="Q55" s="73"/>
     </row>
     <row r="56" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="172">
+      <c r="A56" s="157">
         <v>54</v>
       </c>
-      <c r="B56" s="124"/>
+      <c r="B56" s="168"/>
       <c r="C56" s="79" t="s">
         <v>251</v>
       </c>
@@ -5157,10 +5159,10 @@
       <c r="Q56" s="73"/>
     </row>
     <row r="57" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="172">
+      <c r="A57" s="157">
         <v>55</v>
       </c>
-      <c r="B57" s="124"/>
+      <c r="B57" s="168"/>
       <c r="C57" s="79" t="s">
         <v>252</v>
       </c>
@@ -5191,10 +5193,10 @@
       <c r="Q57" s="73"/>
     </row>
     <row r="58" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="172">
+      <c r="A58" s="157">
         <v>56</v>
       </c>
-      <c r="B58" s="124"/>
+      <c r="B58" s="168"/>
       <c r="C58" s="72"/>
       <c r="D58" s="68"/>
       <c r="E58" s="68"/>
@@ -5223,10 +5225,10 @@
       <c r="Q58" s="73"/>
     </row>
     <row r="59" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="177">
+      <c r="A59" s="162">
         <v>57</v>
       </c>
-      <c r="B59" s="125"/>
+      <c r="B59" s="169"/>
       <c r="C59" s="80" t="s">
         <v>253</v>
       </c>
@@ -5251,7 +5253,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="L59" s="152" t="s">
+      <c r="L59" s="137" t="s">
         <v>246</v>
       </c>
       <c r="M59" s="74"/>
@@ -5261,43 +5263,38 @@
       <c r="Q59" s="77"/>
     </row>
     <row r="60" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J60" s="117" t="s">
+      <c r="J60" s="170" t="s">
         <v>143</v>
       </c>
-      <c r="K60" s="117"/>
-      <c r="L60" s="117"/>
-      <c r="M60" s="117"/>
+      <c r="K60" s="170"/>
+      <c r="L60" s="170"/>
+      <c r="M60" s="170"/>
       <c r="N60" s="23"/>
       <c r="O60" s="24"/>
       <c r="P60" s="25">
         <f>SUM(P3:P59)</f>
-        <v>324.72350000000006</v>
+        <v>334.20349999999996</v>
       </c>
     </row>
     <row r="61" spans="1:17" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="J61" s="118" t="s">
+      <c r="J61" s="171" t="s">
         <v>144</v>
       </c>
-      <c r="K61" s="118"/>
-      <c r="L61" s="118"/>
-      <c r="M61" s="118"/>
+      <c r="K61" s="171"/>
+      <c r="L61" s="171"/>
+      <c r="M61" s="171"/>
       <c r="N61" s="26">
         <f>SUM(N3:N60)</f>
-        <v>70.299900000000008</v>
+        <v>72.469900000000024</v>
       </c>
       <c r="O61" s="27"/>
       <c r="P61" s="26">
         <f>P60/5</f>
-        <v>64.944700000000012</v>
+        <v>66.840699999999998</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B23:B35"/>
-    <mergeCell ref="B37:B45"/>
-    <mergeCell ref="B46:B52"/>
-    <mergeCell ref="B53:B59"/>
-    <mergeCell ref="J60:M60"/>
     <mergeCell ref="J61:M61"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="B3:B10"/>
@@ -5305,6 +5302,11 @@
     <mergeCell ref="B14:B17"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="B20:B22"/>
+    <mergeCell ref="B23:B35"/>
+    <mergeCell ref="B37:B45"/>
+    <mergeCell ref="B46:B52"/>
+    <mergeCell ref="B53:B59"/>
+    <mergeCell ref="J60:M60"/>
   </mergeCells>
   <conditionalFormatting sqref="N61">
     <cfRule type="dataBar" priority="22">
@@ -5667,76 +5669,76 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G6" r:id="rId3" display="https://lcsc.com/brand-detail/392.html"/>
-    <hyperlink ref="G7" r:id="rId4" display="https://lcsc.com/brand-detail/254.html"/>
-    <hyperlink ref="G12" r:id="rId5" display="https://lcsc.com/brand-detail/296.html"/>
-    <hyperlink ref="G21" r:id="rId6" display="https://lcsc.com/brand-detail/94.html"/>
-    <hyperlink ref="G41" r:id="rId7" display="https://lcsc.com/brand-detail/756.html"/>
-    <hyperlink ref="G42" r:id="rId8" display="https://lcsc.com/brand-detail/100.html"/>
-    <hyperlink ref="G50" r:id="rId9" display="https://lcsc.com/brand-detail/109.html"/>
-    <hyperlink ref="L3" r:id="rId10"/>
-    <hyperlink ref="L4" r:id="rId11"/>
-    <hyperlink ref="L7" r:id="rId12"/>
-    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html"/>
-    <hyperlink ref="L11" r:id="rId14"/>
-    <hyperlink ref="G11" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/central-semiconductor"/>
-    <hyperlink ref="L12" r:id="rId16"/>
-    <hyperlink ref="G17" r:id="rId17" display="https://www.digikey.com/en/supplier-centers/sunled"/>
-    <hyperlink ref="L17" r:id="rId18"/>
-    <hyperlink ref="G18" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/wurth-electronics"/>
-    <hyperlink ref="L18" r:id="rId20"/>
-    <hyperlink ref="G20" r:id="rId21" display="https://lcsc.com/brand-detail/296.html"/>
-    <hyperlink ref="G19" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/tdk"/>
-    <hyperlink ref="L20" r:id="rId23"/>
-    <hyperlink ref="L21" r:id="rId24"/>
-    <hyperlink ref="G39" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/texas-instruments"/>
-    <hyperlink ref="G38" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics"/>
-    <hyperlink ref="L38" r:id="rId27"/>
-    <hyperlink ref="L42" r:id="rId28"/>
-    <hyperlink ref="G43" r:id="rId29" display="https://www.digikey.com/en/supplier-centers/analog-devices"/>
-    <hyperlink ref="L43" r:id="rId30"/>
-    <hyperlink ref="L50" r:id="rId31"/>
-    <hyperlink ref="L8" r:id="rId32"/>
-    <hyperlink ref="L39" r:id="rId33"/>
-    <hyperlink ref="L41" r:id="rId34"/>
-    <hyperlink ref="L13" r:id="rId35"/>
-    <hyperlink ref="L22" r:id="rId36"/>
-    <hyperlink ref="L36" r:id="rId37"/>
-    <hyperlink ref="G37" r:id="rId38" display="https://lcsc.com/brand-detail/877.html"/>
-    <hyperlink ref="L40" r:id="rId39"/>
-    <hyperlink ref="L44" r:id="rId40"/>
-    <hyperlink ref="L45" r:id="rId41"/>
-    <hyperlink ref="L5" r:id="rId42"/>
-    <hyperlink ref="L14" r:id="rId43"/>
-    <hyperlink ref="L10" r:id="rId44"/>
-    <hyperlink ref="L53" r:id="rId45"/>
-    <hyperlink ref="L54" r:id="rId46" location="customerReviews"/>
-    <hyperlink ref="L57" r:id="rId47"/>
-    <hyperlink ref="L55" r:id="rId48"/>
-    <hyperlink ref="L59" r:id="rId49"/>
-    <hyperlink ref="L37" r:id="rId50"/>
-    <hyperlink ref="L23" r:id="rId51"/>
-    <hyperlink ref="L24" r:id="rId52"/>
-    <hyperlink ref="L25" r:id="rId53"/>
-    <hyperlink ref="L26" r:id="rId54"/>
-    <hyperlink ref="L27" r:id="rId55"/>
-    <hyperlink ref="L29" r:id="rId56"/>
-    <hyperlink ref="L28" r:id="rId57"/>
-    <hyperlink ref="L30" r:id="rId58"/>
-    <hyperlink ref="L31" r:id="rId59"/>
-    <hyperlink ref="L33" r:id="rId60"/>
-    <hyperlink ref="L34" r:id="rId61"/>
-    <hyperlink ref="L35" r:id="rId62"/>
-    <hyperlink ref="L32" r:id="rId63"/>
-    <hyperlink ref="L6" r:id="rId64"/>
-    <hyperlink ref="L9" r:id="rId65"/>
-    <hyperlink ref="L19" r:id="rId66"/>
-    <hyperlink ref="L46" r:id="rId67"/>
-    <hyperlink ref="L47" r:id="rId68"/>
-    <hyperlink ref="L48" r:id="rId69"/>
-    <hyperlink ref="L49" r:id="rId70"/>
+    <hyperlink ref="G3" r:id="rId1" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G4" r:id="rId2" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="G6" r:id="rId3" display="https://lcsc.com/brand-detail/392.html" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G7" r:id="rId4" display="https://lcsc.com/brand-detail/254.html" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="G12" r:id="rId5" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="G21" r:id="rId6" display="https://lcsc.com/brand-detail/94.html" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G41" r:id="rId7" display="https://lcsc.com/brand-detail/756.html" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="G42" r:id="rId8" display="https://lcsc.com/brand-detail/100.html" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="G50" r:id="rId9" display="https://lcsc.com/brand-detail/109.html" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="L3" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="L4" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="L7" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="G8" r:id="rId13" display="https://lcsc.com/brand-detail/994.html" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="L11" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="G11" r:id="rId15" display="https://www.digikey.com/en/supplier-centers/central-semiconductor" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="L12" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="G17" r:id="rId17" display="https://www.digikey.com/en/supplier-centers/sunled" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="L17" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="G18" r:id="rId19" display="https://www.digikey.com/en/supplier-centers/wurth-electronics" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="L18" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="G20" r:id="rId21" display="https://lcsc.com/brand-detail/296.html" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="G19" r:id="rId22" display="https://www.digikey.com/en/supplier-centers/tdk" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="L20" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="L21" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="G39" r:id="rId25" display="https://www.digikey.com/en/supplier-centers/texas-instruments" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="G38" r:id="rId26" display="https://www.digikey.com/en/supplier-centers/stmicroelectronics" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="L38" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="L42" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="G43" r:id="rId29" display="https://www.digikey.com/en/supplier-centers/analog-devices" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="L43" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="L50" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="L8" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="L39" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="L41" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="L13" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="L22" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="L36" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="G37" r:id="rId38" display="https://lcsc.com/brand-detail/877.html" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="L40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="L44" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="L45" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="L5" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="L14" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="L10" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="L53" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="L54" r:id="rId46" location="customerReviews" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="L57" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="L55" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="L59" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="L37" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="L23" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="L24" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="L25" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="L26" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="L27" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="L29" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="L28" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="L30" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="L31" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="L33" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="L34" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="L35" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="L32" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="L6" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="L9" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="L19" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="L46" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="L47" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="L48" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="L49" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId71"/>

</xml_diff>